<commit_message>
Aplicar formula oficial de direccion de Forecast Accuracy con nueva columna en Excels y App Web
</commit_message>
<xml_diff>
--- a/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_Alfonso.xlsx
+++ b/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_Alfonso.xlsx
@@ -738,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:U44"/>
+  <dimension ref="B2:V44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -749,19 +749,20 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -774,14 +775,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DELEGADO COMERCIAL: ALFONSO | Cierre Septiembre Oficial (01/10/2026) vs Previsiones a Final de Año | Generado: 01/10/2026 10:17</t>
+          <t>DELEGADO COMERCIAL: ALFONSO | Cierre Septiembre Oficial (01/10/2026) vs Previsiones a Final de Año | Generado: 01/10/2026 10:45</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>📌 INSTRUCCIONES: 1) Revise el bloque de SEPTIEMBRE (Previsto vs Real) e indique en la col. K el motivo de la desviación (adelanto, atraso, extra). 2) En las columnas verdes (M, O, Q), revise y actualice las cantidades estimadas de Octubre, Noviembre y Diciembre si prevé cambios. 3) Comente en col. U cualquier nota de campaña.</t>
+          <t>📌 INSTRUCCIONES: 1) Revise el bloque de SEPTIEMBRE (Previsto, Real, Error Absoluto y Forecast Accuracy) e indique en col. L el motivo de la desviación (adelanto, atraso, extra). 2) En las columnas verdes (N, P, R), revise y actualice las cantidades estimadas de Octubre, Noviembre y Diciembre si prevé cambios. 3) Comente en col. V cualquier nota de campaña.</t>
         </is>
       </c>
     </row>
@@ -808,32 +809,33 @@
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>FORECAST ACCURACY SEP</t>
+          <t>FORECAST ACCURACY SEP (OFICIAL)</t>
         </is>
       </c>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>PREVISIÓN INICIAL Q4 (U)</t>
         </is>
       </c>
-      <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="O5" s="5" t="n"/>
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>PREVISIÓN REVISADA Q4 (U)</t>
         </is>
       </c>
-      <c r="P5" s="5" t="n"/>
       <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="8" t="inlineStr">
+      <c r="R5" s="5" t="n"/>
+      <c r="S5" s="8" t="inlineStr">
         <is>
           <t>VARIACIÓN NETA Q4 (U)</t>
         </is>
       </c>
-      <c r="S5" s="5" t="n"/>
       <c r="T5" s="5" t="n"/>
       <c r="U5" s="5" t="n"/>
+      <c r="V5" s="5" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="B6" s="9">
@@ -849,34 +851,35 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="11">
-        <f>I44</f>
+        <f>J44</f>
         <v/>
       </c>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="11">
-        <f>J44</f>
+        <f>K44</f>
         <v/>
       </c>
       <c r="K6" s="5" t="n"/>
-      <c r="L6" s="9">
-        <f>R44</f>
-        <v/>
-      </c>
-      <c r="M6" s="5" t="n"/>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="9">
+        <f>S44</f>
+        <v/>
+      </c>
       <c r="N6" s="5" t="n"/>
-      <c r="O6" s="10">
-        <f>S44</f>
-        <v/>
-      </c>
-      <c r="P6" s="5" t="n"/>
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="10">
+        <f>T44</f>
+        <v/>
+      </c>
       <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="12">
-        <f>T44</f>
-        <v/>
-      </c>
-      <c r="S6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="12">
+        <f>U44</f>
+        <v/>
+      </c>
       <c r="T6" s="5" t="n"/>
       <c r="U6" s="5" t="n"/>
+      <c r="V6" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="13" t="inlineStr">
@@ -886,15 +889,15 @@
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>CIERRE SEPTIEMBRE 2026 (CALIBRACIÓN Y ANÁLISIS)</t>
-        </is>
-      </c>
-      <c r="L8" s="15" t="inlineStr">
+          <t>CIERRE SEPTIEMBRE 2026 (CALIBRACIÓN Y ANÁLISIS DE EXACTITUD)</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="inlineStr">
         <is>
           <t>REVISIÓN PREVISIONES MES A MES (HASTA FINAL DE AÑO 2026)</t>
         </is>
       </c>
-      <c r="R8" s="16" t="inlineStr">
+      <c r="S8" s="16" t="inlineStr">
         <is>
           <t>IMPACTO Q4 Y JUSTIFICACIÓN</t>
         </is>
@@ -938,65 +941,70 @@
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
+          <t>Error Abs. Sep (u)</t>
+        </is>
+      </c>
+      <c r="J9" s="18" t="inlineStr">
+        <is>
           <t>% Consec.</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr">
+      <c r="K9" s="18" t="inlineStr">
         <is>
           <t>Forecast Accuracy</t>
         </is>
       </c>
-      <c r="K9" s="18" t="inlineStr">
+      <c r="L9" s="18" t="inlineStr">
         <is>
           <t>Comentario Sep (¿Adelanto/Atraso/Extra?)</t>
         </is>
       </c>
-      <c r="L9" s="19" t="inlineStr">
+      <c r="M9" s="19" t="inlineStr">
         <is>
           <t>Oct Anterior (u)</t>
         </is>
       </c>
-      <c r="M9" s="19" t="inlineStr">
+      <c r="N9" s="19" t="inlineStr">
         <is>
           <t>Oct Revisado (u)</t>
         </is>
       </c>
-      <c r="N9" s="19" t="inlineStr">
+      <c r="O9" s="19" t="inlineStr">
         <is>
           <t>Nov Anterior (u)</t>
         </is>
       </c>
-      <c r="O9" s="19" t="inlineStr">
+      <c r="P9" s="19" t="inlineStr">
         <is>
           <t>Nov Revisado (u)</t>
         </is>
       </c>
-      <c r="P9" s="19" t="inlineStr">
+      <c r="Q9" s="19" t="inlineStr">
         <is>
           <t>Dic Anterior (u)</t>
         </is>
       </c>
-      <c r="Q9" s="19" t="inlineStr">
+      <c r="R9" s="19" t="inlineStr">
         <is>
           <t>Dic Revisado (u)</t>
         </is>
       </c>
-      <c r="R9" s="17" t="inlineStr">
+      <c r="S9" s="17" t="inlineStr">
         <is>
           <t>Total Q4 Ant (u)</t>
         </is>
       </c>
-      <c r="S9" s="17" t="inlineStr">
+      <c r="T9" s="17" t="inlineStr">
         <is>
           <t>Total Q4 Rev (u)</t>
         </is>
       </c>
-      <c r="T9" s="17" t="inlineStr">
+      <c r="U9" s="17" t="inlineStr">
         <is>
           <t>Dif Q4 (u)</t>
         </is>
       </c>
-      <c r="U9" s="17" t="inlineStr">
+      <c r="V9" s="17" t="inlineStr">
         <is>
           <t>Comentarios / Justificación Q4</t>
         </is>
@@ -1033,46 +1041,50 @@
         <f>G10-F10</f>
         <v/>
       </c>
-      <c r="I10" s="26">
+      <c r="I10" s="23">
+        <f>ABS(G10-F10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="26">
         <f>IF(F10&gt;0, G10/F10, IF(G10&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J10" s="27">
-        <f>IF(F10=0, IF(G10=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G10-F10)/F10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="28" t="inlineStr"/>
-      <c r="L10" s="29" t="n">
+      <c r="K10" s="27">
+        <f>IF(F10&gt;0, 1.0 - (I10/F10), IF(G10=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L10" s="28" t="inlineStr"/>
+      <c r="M10" s="29" t="n">
         <v>960</v>
       </c>
-      <c r="M10" s="30" t="n">
+      <c r="N10" s="30" t="n">
         <v>960</v>
       </c>
-      <c r="N10" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="29" t="n">
+      <c r="O10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="29" t="n">
         <v>960</v>
       </c>
-      <c r="Q10" s="30" t="n">
+      <c r="R10" s="30" t="n">
         <v>960</v>
       </c>
-      <c r="R10" s="23">
-        <f>L10+N10+P10</f>
-        <v/>
-      </c>
-      <c r="S10" s="24">
+      <c r="S10" s="23">
         <f>M10+O10+Q10</f>
         <v/>
       </c>
-      <c r="T10" s="25">
-        <f>S10-R10</f>
-        <v/>
-      </c>
-      <c r="U10" s="31" t="inlineStr"/>
+      <c r="T10" s="24">
+        <f>N10+P10+R10</f>
+        <v/>
+      </c>
+      <c r="U10" s="25">
+        <f>T10-S10</f>
+        <v/>
+      </c>
+      <c r="V10" s="31" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="20" t="inlineStr">
@@ -1105,46 +1117,50 @@
         <f>G11-F11</f>
         <v/>
       </c>
-      <c r="I11" s="26">
+      <c r="I11" s="23">
+        <f>ABS(G11-F11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="26">
         <f>IF(F11&gt;0, G11/F11, IF(G11&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J11" s="27">
-        <f>IF(F11=0, IF(G11=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G11-F11)/F11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="29" t="n">
+      <c r="K11" s="27">
+        <f>IF(F11&gt;0, 1.0 - (I11/F11), IF(G11=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L11" s="28" t="inlineStr"/>
+      <c r="M11" s="29" t="n">
         <v>920</v>
       </c>
-      <c r="M11" s="30" t="n">
+      <c r="N11" s="30" t="n">
         <v>920</v>
       </c>
-      <c r="N11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="29" t="n">
+      <c r="O11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="29" t="n">
         <v>960</v>
       </c>
-      <c r="Q11" s="30" t="n">
+      <c r="R11" s="30" t="n">
         <v>960</v>
       </c>
-      <c r="R11" s="23">
-        <f>L11+N11+P11</f>
-        <v/>
-      </c>
-      <c r="S11" s="24">
+      <c r="S11" s="23">
         <f>M11+O11+Q11</f>
         <v/>
       </c>
-      <c r="T11" s="25">
-        <f>S11-R11</f>
-        <v/>
-      </c>
-      <c r="U11" s="31" t="inlineStr"/>
+      <c r="T11" s="24">
+        <f>N11+P11+R11</f>
+        <v/>
+      </c>
+      <c r="U11" s="25">
+        <f>T11-S11</f>
+        <v/>
+      </c>
+      <c r="V11" s="31" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="20" t="inlineStr">
@@ -1177,50 +1193,54 @@
         <f>G12-F12</f>
         <v/>
       </c>
-      <c r="I12" s="26">
+      <c r="I12" s="23">
+        <f>ABS(G12-F12)</f>
+        <v/>
+      </c>
+      <c r="J12" s="26">
         <f>IF(F12&gt;0, G12/F12, IF(G12&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J12" s="27">
-        <f>IF(F12=0, IF(G12=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G12-F12)/F12))</f>
-        <v/>
-      </c>
-      <c r="K12" s="28" t="inlineStr">
+      <c r="K12" s="27">
+        <f>IF(F12&gt;0, 1.0 - (I12/F12), IF(G12=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L12" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="23">
-        <f>L12+N12+P12</f>
-        <v/>
-      </c>
-      <c r="S12" s="24">
+      <c r="M12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="23">
         <f>M12+O12+Q12</f>
         <v/>
       </c>
-      <c r="T12" s="25">
-        <f>S12-R12</f>
-        <v/>
-      </c>
-      <c r="U12" s="31" t="inlineStr"/>
+      <c r="T12" s="24">
+        <f>N12+P12+R12</f>
+        <v/>
+      </c>
+      <c r="U12" s="25">
+        <f>T12-S12</f>
+        <v/>
+      </c>
+      <c r="V12" s="31" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="20" t="inlineStr">
@@ -1253,50 +1273,54 @@
         <f>G13-F13</f>
         <v/>
       </c>
-      <c r="I13" s="26">
+      <c r="I13" s="23">
+        <f>ABS(G13-F13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="26">
         <f>IF(F13&gt;0, G13/F13, IF(G13&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J13" s="27">
-        <f>IF(F13=0, IF(G13=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G13-F13)/F13))</f>
-        <v/>
-      </c>
-      <c r="K13" s="28" t="inlineStr">
+      <c r="K13" s="27">
+        <f>IF(F13&gt;0, 1.0 - (I13/F13), IF(G13=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L13" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="23">
-        <f>L13+N13+P13</f>
-        <v/>
-      </c>
-      <c r="S13" s="24">
+      <c r="M13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="23">
         <f>M13+O13+Q13</f>
         <v/>
       </c>
-      <c r="T13" s="25">
-        <f>S13-R13</f>
-        <v/>
-      </c>
-      <c r="U13" s="31" t="inlineStr"/>
+      <c r="T13" s="24">
+        <f>N13+P13+R13</f>
+        <v/>
+      </c>
+      <c r="U13" s="25">
+        <f>T13-S13</f>
+        <v/>
+      </c>
+      <c r="V13" s="31" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="20" t="inlineStr">
@@ -1329,50 +1353,54 @@
         <f>G14-F14</f>
         <v/>
       </c>
-      <c r="I14" s="26">
+      <c r="I14" s="23">
+        <f>ABS(G14-F14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="26">
         <f>IF(F14&gt;0, G14/F14, IF(G14&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J14" s="27">
-        <f>IF(F14=0, IF(G14=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G14-F14)/F14))</f>
-        <v/>
-      </c>
-      <c r="K14" s="28" t="inlineStr">
+      <c r="K14" s="27">
+        <f>IF(F14&gt;0, 1.0 - (I14/F14), IF(G14=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L14" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="23">
-        <f>L14+N14+P14</f>
-        <v/>
-      </c>
-      <c r="S14" s="24">
+      <c r="M14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="23">
         <f>M14+O14+Q14</f>
         <v/>
       </c>
-      <c r="T14" s="25">
-        <f>S14-R14</f>
-        <v/>
-      </c>
-      <c r="U14" s="31" t="inlineStr"/>
+      <c r="T14" s="24">
+        <f>N14+P14+R14</f>
+        <v/>
+      </c>
+      <c r="U14" s="25">
+        <f>T14-S14</f>
+        <v/>
+      </c>
+      <c r="V14" s="31" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="20" t="inlineStr">
@@ -1405,50 +1433,54 @@
         <f>G15-F15</f>
         <v/>
       </c>
-      <c r="I15" s="26">
+      <c r="I15" s="23">
+        <f>ABS(G15-F15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="26">
         <f>IF(F15&gt;0, G15/F15, IF(G15&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J15" s="27">
-        <f>IF(F15=0, IF(G15=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G15-F15)/F15))</f>
-        <v/>
-      </c>
-      <c r="K15" s="28" t="inlineStr">
+      <c r="K15" s="27">
+        <f>IF(F15&gt;0, 1.0 - (I15/F15), IF(G15=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L15" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="23">
-        <f>L15+N15+P15</f>
-        <v/>
-      </c>
-      <c r="S15" s="24">
+      <c r="M15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="23">
         <f>M15+O15+Q15</f>
         <v/>
       </c>
-      <c r="T15" s="25">
-        <f>S15-R15</f>
-        <v/>
-      </c>
-      <c r="U15" s="31" t="inlineStr"/>
+      <c r="T15" s="24">
+        <f>N15+P15+R15</f>
+        <v/>
+      </c>
+      <c r="U15" s="25">
+        <f>T15-S15</f>
+        <v/>
+      </c>
+      <c r="V15" s="31" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="20" t="inlineStr">
@@ -1481,50 +1513,54 @@
         <f>G16-F16</f>
         <v/>
       </c>
-      <c r="I16" s="26">
+      <c r="I16" s="23">
+        <f>ABS(G16-F16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="26">
         <f>IF(F16&gt;0, G16/F16, IF(G16&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J16" s="27">
-        <f>IF(F16=0, IF(G16=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G16-F16)/F16))</f>
-        <v/>
-      </c>
-      <c r="K16" s="28" t="inlineStr">
+      <c r="K16" s="27">
+        <f>IF(F16&gt;0, 1.0 - (I16/F16), IF(G16=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L16" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="23">
-        <f>L16+N16+P16</f>
-        <v/>
-      </c>
-      <c r="S16" s="24">
+      <c r="M16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="23">
         <f>M16+O16+Q16</f>
         <v/>
       </c>
-      <c r="T16" s="25">
-        <f>S16-R16</f>
-        <v/>
-      </c>
-      <c r="U16" s="31" t="inlineStr"/>
+      <c r="T16" s="24">
+        <f>N16+P16+R16</f>
+        <v/>
+      </c>
+      <c r="U16" s="25">
+        <f>T16-S16</f>
+        <v/>
+      </c>
+      <c r="V16" s="31" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="20" t="inlineStr">
@@ -1557,50 +1593,54 @@
         <f>G17-F17</f>
         <v/>
       </c>
-      <c r="I17" s="26">
+      <c r="I17" s="23">
+        <f>ABS(G17-F17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="26">
         <f>IF(F17&gt;0, G17/F17, IF(G17&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J17" s="27">
-        <f>IF(F17=0, IF(G17=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G17-F17)/F17))</f>
-        <v/>
-      </c>
-      <c r="K17" s="28" t="inlineStr">
+      <c r="K17" s="27">
+        <f>IF(F17&gt;0, 1.0 - (I17/F17), IF(G17=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L17" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="23">
-        <f>L17+N17+P17</f>
-        <v/>
-      </c>
-      <c r="S17" s="24">
+      <c r="M17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="23">
         <f>M17+O17+Q17</f>
         <v/>
       </c>
-      <c r="T17" s="25">
-        <f>S17-R17</f>
-        <v/>
-      </c>
-      <c r="U17" s="31" t="inlineStr"/>
+      <c r="T17" s="24">
+        <f>N17+P17+R17</f>
+        <v/>
+      </c>
+      <c r="U17" s="25">
+        <f>T17-S17</f>
+        <v/>
+      </c>
+      <c r="V17" s="31" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="20" t="inlineStr">
@@ -1633,46 +1673,50 @@
         <f>G18-F18</f>
         <v/>
       </c>
-      <c r="I18" s="26">
+      <c r="I18" s="23">
+        <f>ABS(G18-F18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="26">
         <f>IF(F18&gt;0, G18/F18, IF(G18&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J18" s="27">
-        <f>IF(F18=0, IF(G18=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G18-F18)/F18))</f>
-        <v/>
-      </c>
-      <c r="K18" s="28" t="inlineStr"/>
-      <c r="L18" s="29" t="n">
+      <c r="K18" s="27">
+        <f>IF(F18&gt;0, 1.0 - (I18/F18), IF(G18=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L18" s="28" t="inlineStr"/>
+      <c r="M18" s="29" t="n">
         <v>300</v>
       </c>
-      <c r="M18" s="30" t="n">
+      <c r="N18" s="30" t="n">
         <v>300</v>
       </c>
-      <c r="N18" s="29" t="n">
+      <c r="O18" s="29" t="n">
         <v>400</v>
       </c>
-      <c r="O18" s="30" t="n">
+      <c r="P18" s="30" t="n">
         <v>400</v>
       </c>
-      <c r="P18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="23">
-        <f>L18+N18+P18</f>
-        <v/>
-      </c>
-      <c r="S18" s="24">
+      <c r="Q18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="23">
         <f>M18+O18+Q18</f>
         <v/>
       </c>
-      <c r="T18" s="25">
-        <f>S18-R18</f>
-        <v/>
-      </c>
-      <c r="U18" s="31" t="inlineStr"/>
+      <c r="T18" s="24">
+        <f>N18+P18+R18</f>
+        <v/>
+      </c>
+      <c r="U18" s="25">
+        <f>T18-S18</f>
+        <v/>
+      </c>
+      <c r="V18" s="31" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="20" t="inlineStr">
@@ -1705,46 +1749,50 @@
         <f>G19-F19</f>
         <v/>
       </c>
-      <c r="I19" s="26">
+      <c r="I19" s="23">
+        <f>ABS(G19-F19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="26">
         <f>IF(F19&gt;0, G19/F19, IF(G19&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J19" s="27">
-        <f>IF(F19=0, IF(G19=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G19-F19)/F19))</f>
-        <v/>
-      </c>
-      <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="29" t="n">
+      <c r="K19" s="27">
+        <f>IF(F19&gt;0, 1.0 - (I19/F19), IF(G19=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L19" s="28" t="inlineStr"/>
+      <c r="M19" s="29" t="n">
         <v>640</v>
       </c>
-      <c r="M19" s="30" t="n">
+      <c r="N19" s="30" t="n">
         <v>640</v>
       </c>
-      <c r="N19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="23">
-        <f>L19+N19+P19</f>
-        <v/>
-      </c>
-      <c r="S19" s="24">
+      <c r="O19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="23">
         <f>M19+O19+Q19</f>
         <v/>
       </c>
-      <c r="T19" s="25">
-        <f>S19-R19</f>
-        <v/>
-      </c>
-      <c r="U19" s="31" t="inlineStr"/>
+      <c r="T19" s="24">
+        <f>N19+P19+R19</f>
+        <v/>
+      </c>
+      <c r="U19" s="25">
+        <f>T19-S19</f>
+        <v/>
+      </c>
+      <c r="V19" s="31" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="20" t="inlineStr">
@@ -1777,50 +1825,54 @@
         <f>G20-F20</f>
         <v/>
       </c>
-      <c r="I20" s="26">
+      <c r="I20" s="23">
+        <f>ABS(G20-F20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="26">
         <f>IF(F20&gt;0, G20/F20, IF(G20&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J20" s="27">
-        <f>IF(F20=0, IF(G20=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G20-F20)/F20))</f>
-        <v/>
-      </c>
-      <c r="K20" s="28" t="inlineStr">
+      <c r="K20" s="27">
+        <f>IF(F20&gt;0, 1.0 - (I20/F20), IF(G20=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L20" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="23">
-        <f>L20+N20+P20</f>
-        <v/>
-      </c>
-      <c r="S20" s="24">
+      <c r="M20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="23">
         <f>M20+O20+Q20</f>
         <v/>
       </c>
-      <c r="T20" s="25">
-        <f>S20-R20</f>
-        <v/>
-      </c>
-      <c r="U20" s="31" t="inlineStr"/>
+      <c r="T20" s="24">
+        <f>N20+P20+R20</f>
+        <v/>
+      </c>
+      <c r="U20" s="25">
+        <f>T20-S20</f>
+        <v/>
+      </c>
+      <c r="V20" s="31" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="20" t="inlineStr">
@@ -1853,50 +1905,54 @@
         <f>G21-F21</f>
         <v/>
       </c>
-      <c r="I21" s="26">
+      <c r="I21" s="23">
+        <f>ABS(G21-F21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="26">
         <f>IF(F21&gt;0, G21/F21, IF(G21&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J21" s="27">
-        <f>IF(F21=0, IF(G21=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G21-F21)/F21))</f>
-        <v/>
-      </c>
-      <c r="K21" s="28" t="inlineStr">
+      <c r="K21" s="27">
+        <f>IF(F21&gt;0, 1.0 - (I21/F21), IF(G21=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L21" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="23">
-        <f>L21+N21+P21</f>
-        <v/>
-      </c>
-      <c r="S21" s="24">
+      <c r="M21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="23">
         <f>M21+O21+Q21</f>
         <v/>
       </c>
-      <c r="T21" s="25">
-        <f>S21-R21</f>
-        <v/>
-      </c>
-      <c r="U21" s="31" t="inlineStr"/>
+      <c r="T21" s="24">
+        <f>N21+P21+R21</f>
+        <v/>
+      </c>
+      <c r="U21" s="25">
+        <f>T21-S21</f>
+        <v/>
+      </c>
+      <c r="V21" s="31" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="20" t="inlineStr">
@@ -1929,50 +1985,54 @@
         <f>G22-F22</f>
         <v/>
       </c>
-      <c r="I22" s="26">
+      <c r="I22" s="23">
+        <f>ABS(G22-F22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="26">
         <f>IF(F22&gt;0, G22/F22, IF(G22&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J22" s="27">
-        <f>IF(F22=0, IF(G22=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G22-F22)/F22))</f>
-        <v/>
-      </c>
-      <c r="K22" s="28" t="inlineStr">
+      <c r="K22" s="27">
+        <f>IF(F22&gt;0, 1.0 - (I22/F22), IF(G22=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L22" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="23">
-        <f>L22+N22+P22</f>
-        <v/>
-      </c>
-      <c r="S22" s="24">
+      <c r="M22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="23">
         <f>M22+O22+Q22</f>
         <v/>
       </c>
-      <c r="T22" s="25">
-        <f>S22-R22</f>
-        <v/>
-      </c>
-      <c r="U22" s="31" t="inlineStr"/>
+      <c r="T22" s="24">
+        <f>N22+P22+R22</f>
+        <v/>
+      </c>
+      <c r="U22" s="25">
+        <f>T22-S22</f>
+        <v/>
+      </c>
+      <c r="V22" s="31" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="20" t="inlineStr">
@@ -2005,50 +2065,54 @@
         <f>G23-F23</f>
         <v/>
       </c>
-      <c r="I23" s="26">
+      <c r="I23" s="23">
+        <f>ABS(G23-F23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="26">
         <f>IF(F23&gt;0, G23/F23, IF(G23&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J23" s="27">
-        <f>IF(F23=0, IF(G23=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G23-F23)/F23))</f>
-        <v/>
-      </c>
-      <c r="K23" s="28" t="inlineStr">
+      <c r="K23" s="27">
+        <f>IF(F23&gt;0, 1.0 - (I23/F23), IF(G23=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L23" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="23">
-        <f>L23+N23+P23</f>
-        <v/>
-      </c>
-      <c r="S23" s="24">
+      <c r="M23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="23">
         <f>M23+O23+Q23</f>
         <v/>
       </c>
-      <c r="T23" s="25">
-        <f>S23-R23</f>
-        <v/>
-      </c>
-      <c r="U23" s="31" t="inlineStr"/>
+      <c r="T23" s="24">
+        <f>N23+P23+R23</f>
+        <v/>
+      </c>
+      <c r="U23" s="25">
+        <f>T23-S23</f>
+        <v/>
+      </c>
+      <c r="V23" s="31" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="20" t="inlineStr">
@@ -2081,50 +2145,54 @@
         <f>G24-F24</f>
         <v/>
       </c>
-      <c r="I24" s="26">
+      <c r="I24" s="23">
+        <f>ABS(G24-F24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="26">
         <f>IF(F24&gt;0, G24/F24, IF(G24&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J24" s="27">
-        <f>IF(F24=0, IF(G24=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G24-F24)/F24))</f>
-        <v/>
-      </c>
-      <c r="K24" s="28" t="inlineStr">
+      <c r="K24" s="27">
+        <f>IF(F24&gt;0, 1.0 - (I24/F24), IF(G24=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L24" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="23">
-        <f>L24+N24+P24</f>
-        <v/>
-      </c>
-      <c r="S24" s="24">
+      <c r="M24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="23">
         <f>M24+O24+Q24</f>
         <v/>
       </c>
-      <c r="T24" s="25">
-        <f>S24-R24</f>
-        <v/>
-      </c>
-      <c r="U24" s="31" t="inlineStr"/>
+      <c r="T24" s="24">
+        <f>N24+P24+R24</f>
+        <v/>
+      </c>
+      <c r="U24" s="25">
+        <f>T24-S24</f>
+        <v/>
+      </c>
+      <c r="V24" s="31" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="20" t="inlineStr">
@@ -2157,50 +2225,54 @@
         <f>G25-F25</f>
         <v/>
       </c>
-      <c r="I25" s="26">
+      <c r="I25" s="23">
+        <f>ABS(G25-F25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="26">
         <f>IF(F25&gt;0, G25/F25, IF(G25&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J25" s="27">
-        <f>IF(F25=0, IF(G25=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G25-F25)/F25))</f>
-        <v/>
-      </c>
-      <c r="K25" s="28" t="inlineStr">
+      <c r="K25" s="27">
+        <f>IF(F25&gt;0, 1.0 - (I25/F25), IF(G25=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L25" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="23">
-        <f>L25+N25+P25</f>
-        <v/>
-      </c>
-      <c r="S25" s="24">
+      <c r="M25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="23">
         <f>M25+O25+Q25</f>
         <v/>
       </c>
-      <c r="T25" s="25">
-        <f>S25-R25</f>
-        <v/>
-      </c>
-      <c r="U25" s="31" t="inlineStr"/>
+      <c r="T25" s="24">
+        <f>N25+P25+R25</f>
+        <v/>
+      </c>
+      <c r="U25" s="25">
+        <f>T25-S25</f>
+        <v/>
+      </c>
+      <c r="V25" s="31" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="20" t="inlineStr">
@@ -2233,50 +2305,54 @@
         <f>G26-F26</f>
         <v/>
       </c>
-      <c r="I26" s="26">
+      <c r="I26" s="23">
+        <f>ABS(G26-F26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="26">
         <f>IF(F26&gt;0, G26/F26, IF(G26&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J26" s="27">
-        <f>IF(F26=0, IF(G26=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G26-F26)/F26))</f>
-        <v/>
-      </c>
-      <c r="K26" s="28" t="inlineStr">
+      <c r="K26" s="27">
+        <f>IF(F26&gt;0, 1.0 - (I26/F26), IF(G26=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="23">
-        <f>L26+N26+P26</f>
-        <v/>
-      </c>
-      <c r="S26" s="24">
+      <c r="M26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="23">
         <f>M26+O26+Q26</f>
         <v/>
       </c>
-      <c r="T26" s="25">
-        <f>S26-R26</f>
-        <v/>
-      </c>
-      <c r="U26" s="31" t="inlineStr"/>
+      <c r="T26" s="24">
+        <f>N26+P26+R26</f>
+        <v/>
+      </c>
+      <c r="U26" s="25">
+        <f>T26-S26</f>
+        <v/>
+      </c>
+      <c r="V26" s="31" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="B27" s="20" t="inlineStr">
@@ -2309,50 +2385,54 @@
         <f>G27-F27</f>
         <v/>
       </c>
-      <c r="I27" s="26">
+      <c r="I27" s="23">
+        <f>ABS(G27-F27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="26">
         <f>IF(F27&gt;0, G27/F27, IF(G27&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J27" s="27">
-        <f>IF(F27=0, IF(G27=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G27-F27)/F27))</f>
-        <v/>
-      </c>
-      <c r="K27" s="28" t="inlineStr">
+      <c r="K27" s="27">
+        <f>IF(F27&gt;0, 1.0 - (I27/F27), IF(G27=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L27" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="23">
-        <f>L27+N27+P27</f>
-        <v/>
-      </c>
-      <c r="S27" s="24">
+      <c r="M27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="23">
         <f>M27+O27+Q27</f>
         <v/>
       </c>
-      <c r="T27" s="25">
-        <f>S27-R27</f>
-        <v/>
-      </c>
-      <c r="U27" s="31" t="inlineStr"/>
+      <c r="T27" s="24">
+        <f>N27+P27+R27</f>
+        <v/>
+      </c>
+      <c r="U27" s="25">
+        <f>T27-S27</f>
+        <v/>
+      </c>
+      <c r="V27" s="31" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="20" t="inlineStr">
@@ -2385,50 +2465,54 @@
         <f>G28-F28</f>
         <v/>
       </c>
-      <c r="I28" s="26">
+      <c r="I28" s="23">
+        <f>ABS(G28-F28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="26">
         <f>IF(F28&gt;0, G28/F28, IF(G28&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J28" s="27">
-        <f>IF(F28=0, IF(G28=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G28-F28)/F28))</f>
-        <v/>
-      </c>
-      <c r="K28" s="28" t="inlineStr">
+      <c r="K28" s="27">
+        <f>IF(F28&gt;0, 1.0 - (I28/F28), IF(G28=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L28" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="23">
-        <f>L28+N28+P28</f>
-        <v/>
-      </c>
-      <c r="S28" s="24">
+      <c r="M28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="23">
         <f>M28+O28+Q28</f>
         <v/>
       </c>
-      <c r="T28" s="25">
-        <f>S28-R28</f>
-        <v/>
-      </c>
-      <c r="U28" s="31" t="inlineStr"/>
+      <c r="T28" s="24">
+        <f>N28+P28+R28</f>
+        <v/>
+      </c>
+      <c r="U28" s="25">
+        <f>T28-S28</f>
+        <v/>
+      </c>
+      <c r="V28" s="31" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="20" t="inlineStr">
@@ -2461,50 +2545,54 @@
         <f>G29-F29</f>
         <v/>
       </c>
-      <c r="I29" s="26">
+      <c r="I29" s="23">
+        <f>ABS(G29-F29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="26">
         <f>IF(F29&gt;0, G29/F29, IF(G29&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J29" s="27">
-        <f>IF(F29=0, IF(G29=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G29-F29)/F29))</f>
-        <v/>
-      </c>
-      <c r="K29" s="28" t="inlineStr">
+      <c r="K29" s="27">
+        <f>IF(F29&gt;0, 1.0 - (I29/F29), IF(G29=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L29" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="23">
-        <f>L29+N29+P29</f>
-        <v/>
-      </c>
-      <c r="S29" s="24">
+      <c r="M29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="23">
         <f>M29+O29+Q29</f>
         <v/>
       </c>
-      <c r="T29" s="25">
-        <f>S29-R29</f>
-        <v/>
-      </c>
-      <c r="U29" s="31" t="inlineStr"/>
+      <c r="T29" s="24">
+        <f>N29+P29+R29</f>
+        <v/>
+      </c>
+      <c r="U29" s="25">
+        <f>T29-S29</f>
+        <v/>
+      </c>
+      <c r="V29" s="31" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="20" t="inlineStr">
@@ -2537,50 +2625,54 @@
         <f>G30-F30</f>
         <v/>
       </c>
-      <c r="I30" s="26">
+      <c r="I30" s="23">
+        <f>ABS(G30-F30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="26">
         <f>IF(F30&gt;0, G30/F30, IF(G30&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J30" s="27">
-        <f>IF(F30=0, IF(G30=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G30-F30)/F30))</f>
-        <v/>
-      </c>
-      <c r="K30" s="28" t="inlineStr">
+      <c r="K30" s="27">
+        <f>IF(F30&gt;0, 1.0 - (I30/F30), IF(G30=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L30" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L30" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="23">
-        <f>L30+N30+P30</f>
-        <v/>
-      </c>
-      <c r="S30" s="24">
+      <c r="M30" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="23">
         <f>M30+O30+Q30</f>
         <v/>
       </c>
-      <c r="T30" s="25">
-        <f>S30-R30</f>
-        <v/>
-      </c>
-      <c r="U30" s="31" t="inlineStr"/>
+      <c r="T30" s="24">
+        <f>N30+P30+R30</f>
+        <v/>
+      </c>
+      <c r="U30" s="25">
+        <f>T30-S30</f>
+        <v/>
+      </c>
+      <c r="V30" s="31" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="20" t="inlineStr">
@@ -2613,50 +2705,54 @@
         <f>G31-F31</f>
         <v/>
       </c>
-      <c r="I31" s="26">
+      <c r="I31" s="23">
+        <f>ABS(G31-F31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="26">
         <f>IF(F31&gt;0, G31/F31, IF(G31&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J31" s="27">
-        <f>IF(F31=0, IF(G31=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G31-F31)/F31))</f>
-        <v/>
-      </c>
-      <c r="K31" s="28" t="inlineStr">
+      <c r="K31" s="27">
+        <f>IF(F31&gt;0, 1.0 - (I31/F31), IF(G31=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L31" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L31" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="23">
-        <f>L31+N31+P31</f>
-        <v/>
-      </c>
-      <c r="S31" s="24">
+      <c r="M31" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="23">
         <f>M31+O31+Q31</f>
         <v/>
       </c>
-      <c r="T31" s="25">
-        <f>S31-R31</f>
-        <v/>
-      </c>
-      <c r="U31" s="31" t="inlineStr"/>
+      <c r="T31" s="24">
+        <f>N31+P31+R31</f>
+        <v/>
+      </c>
+      <c r="U31" s="25">
+        <f>T31-S31</f>
+        <v/>
+      </c>
+      <c r="V31" s="31" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="20" t="inlineStr">
@@ -2689,50 +2785,54 @@
         <f>G32-F32</f>
         <v/>
       </c>
-      <c r="I32" s="26">
+      <c r="I32" s="23">
+        <f>ABS(G32-F32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="26">
         <f>IF(F32&gt;0, G32/F32, IF(G32&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J32" s="27">
-        <f>IF(F32=0, IF(G32=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G32-F32)/F32))</f>
-        <v/>
-      </c>
-      <c r="K32" s="28" t="inlineStr">
+      <c r="K32" s="27">
+        <f>IF(F32&gt;0, 1.0 - (I32/F32), IF(G32=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L32" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L32" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="23">
-        <f>L32+N32+P32</f>
-        <v/>
-      </c>
-      <c r="S32" s="24">
+      <c r="M32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="23">
         <f>M32+O32+Q32</f>
         <v/>
       </c>
-      <c r="T32" s="25">
-        <f>S32-R32</f>
-        <v/>
-      </c>
-      <c r="U32" s="31" t="inlineStr"/>
+      <c r="T32" s="24">
+        <f>N32+P32+R32</f>
+        <v/>
+      </c>
+      <c r="U32" s="25">
+        <f>T32-S32</f>
+        <v/>
+      </c>
+      <c r="V32" s="31" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="20" t="inlineStr">
@@ -2765,50 +2865,54 @@
         <f>G33-F33</f>
         <v/>
       </c>
-      <c r="I33" s="26">
+      <c r="I33" s="23">
+        <f>ABS(G33-F33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="26">
         <f>IF(F33&gt;0, G33/F33, IF(G33&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J33" s="27">
-        <f>IF(F33=0, IF(G33=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G33-F33)/F33))</f>
-        <v/>
-      </c>
-      <c r="K33" s="28" t="inlineStr">
+      <c r="K33" s="27">
+        <f>IF(F33&gt;0, 1.0 - (I33/F33), IF(G33=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L33" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="23">
-        <f>L33+N33+P33</f>
-        <v/>
-      </c>
-      <c r="S33" s="24">
+      <c r="M33" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="23">
         <f>M33+O33+Q33</f>
         <v/>
       </c>
-      <c r="T33" s="25">
-        <f>S33-R33</f>
-        <v/>
-      </c>
-      <c r="U33" s="31" t="inlineStr"/>
+      <c r="T33" s="24">
+        <f>N33+P33+R33</f>
+        <v/>
+      </c>
+      <c r="U33" s="25">
+        <f>T33-S33</f>
+        <v/>
+      </c>
+      <c r="V33" s="31" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="20" t="inlineStr">
@@ -2841,50 +2945,54 @@
         <f>G34-F34</f>
         <v/>
       </c>
-      <c r="I34" s="26">
+      <c r="I34" s="23">
+        <f>ABS(G34-F34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="26">
         <f>IF(F34&gt;0, G34/F34, IF(G34&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J34" s="27">
-        <f>IF(F34=0, IF(G34=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G34-F34)/F34))</f>
-        <v/>
-      </c>
-      <c r="K34" s="28" t="inlineStr">
+      <c r="K34" s="27">
+        <f>IF(F34&gt;0, 1.0 - (I34/F34), IF(G34=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L34" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" s="23">
-        <f>L34+N34+P34</f>
-        <v/>
-      </c>
-      <c r="S34" s="24">
+      <c r="M34" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="23">
         <f>M34+O34+Q34</f>
         <v/>
       </c>
-      <c r="T34" s="25">
-        <f>S34-R34</f>
-        <v/>
-      </c>
-      <c r="U34" s="31" t="inlineStr"/>
+      <c r="T34" s="24">
+        <f>N34+P34+R34</f>
+        <v/>
+      </c>
+      <c r="U34" s="25">
+        <f>T34-S34</f>
+        <v/>
+      </c>
+      <c r="V34" s="31" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="20" t="inlineStr">
@@ -2917,50 +3025,54 @@
         <f>G35-F35</f>
         <v/>
       </c>
-      <c r="I35" s="26">
+      <c r="I35" s="23">
+        <f>ABS(G35-F35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="26">
         <f>IF(F35&gt;0, G35/F35, IF(G35&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J35" s="27">
-        <f>IF(F35=0, IF(G35=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G35-F35)/F35))</f>
-        <v/>
-      </c>
-      <c r="K35" s="28" t="inlineStr">
+      <c r="K35" s="27">
+        <f>IF(F35&gt;0, 1.0 - (I35/F35), IF(G35=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L35" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="23">
-        <f>L35+N35+P35</f>
-        <v/>
-      </c>
-      <c r="S35" s="24">
+      <c r="M35" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="23">
         <f>M35+O35+Q35</f>
         <v/>
       </c>
-      <c r="T35" s="25">
-        <f>S35-R35</f>
-        <v/>
-      </c>
-      <c r="U35" s="31" t="inlineStr"/>
+      <c r="T35" s="24">
+        <f>N35+P35+R35</f>
+        <v/>
+      </c>
+      <c r="U35" s="25">
+        <f>T35-S35</f>
+        <v/>
+      </c>
+      <c r="V35" s="31" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="20" t="inlineStr">
@@ -2993,50 +3105,54 @@
         <f>G36-F36</f>
         <v/>
       </c>
-      <c r="I36" s="26">
+      <c r="I36" s="23">
+        <f>ABS(G36-F36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="26">
         <f>IF(F36&gt;0, G36/F36, IF(G36&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J36" s="27">
-        <f>IF(F36=0, IF(G36=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G36-F36)/F36))</f>
-        <v/>
-      </c>
-      <c r="K36" s="28" t="inlineStr">
+      <c r="K36" s="27">
+        <f>IF(F36&gt;0, 1.0 - (I36/F36), IF(G36=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L36" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L36" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" s="23">
-        <f>L36+N36+P36</f>
-        <v/>
-      </c>
-      <c r="S36" s="24">
+      <c r="M36" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="23">
         <f>M36+O36+Q36</f>
         <v/>
       </c>
-      <c r="T36" s="25">
-        <f>S36-R36</f>
-        <v/>
-      </c>
-      <c r="U36" s="31" t="inlineStr"/>
+      <c r="T36" s="24">
+        <f>N36+P36+R36</f>
+        <v/>
+      </c>
+      <c r="U36" s="25">
+        <f>T36-S36</f>
+        <v/>
+      </c>
+      <c r="V36" s="31" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="20" t="inlineStr">
@@ -3069,50 +3185,54 @@
         <f>G37-F37</f>
         <v/>
       </c>
-      <c r="I37" s="26">
+      <c r="I37" s="23">
+        <f>ABS(G37-F37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="26">
         <f>IF(F37&gt;0, G37/F37, IF(G37&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J37" s="27">
-        <f>IF(F37=0, IF(G37=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G37-F37)/F37))</f>
-        <v/>
-      </c>
-      <c r="K37" s="28" t="inlineStr">
+      <c r="K37" s="27">
+        <f>IF(F37&gt;0, 1.0 - (I37/F37), IF(G37=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L37" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L37" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" s="23">
-        <f>L37+N37+P37</f>
-        <v/>
-      </c>
-      <c r="S37" s="24">
+      <c r="M37" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="23">
         <f>M37+O37+Q37</f>
         <v/>
       </c>
-      <c r="T37" s="25">
-        <f>S37-R37</f>
-        <v/>
-      </c>
-      <c r="U37" s="31" t="inlineStr"/>
+      <c r="T37" s="24">
+        <f>N37+P37+R37</f>
+        <v/>
+      </c>
+      <c r="U37" s="25">
+        <f>T37-S37</f>
+        <v/>
+      </c>
+      <c r="V37" s="31" t="inlineStr"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="20" t="inlineStr">
@@ -3145,50 +3265,54 @@
         <f>G38-F38</f>
         <v/>
       </c>
-      <c r="I38" s="26">
+      <c r="I38" s="23">
+        <f>ABS(G38-F38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="26">
         <f>IF(F38&gt;0, G38/F38, IF(G38&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J38" s="27">
-        <f>IF(F38=0, IF(G38=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G38-F38)/F38))</f>
-        <v/>
-      </c>
-      <c r="K38" s="28" t="inlineStr">
+      <c r="K38" s="27">
+        <f>IF(F38&gt;0, 1.0 - (I38/F38), IF(G38=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L38" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L38" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R38" s="23">
-        <f>L38+N38+P38</f>
-        <v/>
-      </c>
-      <c r="S38" s="24">
+      <c r="M38" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="23">
         <f>M38+O38+Q38</f>
         <v/>
       </c>
-      <c r="T38" s="25">
-        <f>S38-R38</f>
-        <v/>
-      </c>
-      <c r="U38" s="31" t="inlineStr"/>
+      <c r="T38" s="24">
+        <f>N38+P38+R38</f>
+        <v/>
+      </c>
+      <c r="U38" s="25">
+        <f>T38-S38</f>
+        <v/>
+      </c>
+      <c r="V38" s="31" t="inlineStr"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="20" t="inlineStr">
@@ -3221,50 +3345,54 @@
         <f>G39-F39</f>
         <v/>
       </c>
-      <c r="I39" s="26">
+      <c r="I39" s="23">
+        <f>ABS(G39-F39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="26">
         <f>IF(F39&gt;0, G39/F39, IF(G39&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J39" s="27">
-        <f>IF(F39=0, IF(G39=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G39-F39)/F39))</f>
-        <v/>
-      </c>
-      <c r="K39" s="28" t="inlineStr">
+      <c r="K39" s="27">
+        <f>IF(F39&gt;0, 1.0 - (I39/F39), IF(G39=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L39" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L39" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="23">
-        <f>L39+N39+P39</f>
-        <v/>
-      </c>
-      <c r="S39" s="24">
+      <c r="M39" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" s="23">
         <f>M39+O39+Q39</f>
         <v/>
       </c>
-      <c r="T39" s="25">
-        <f>S39-R39</f>
-        <v/>
-      </c>
-      <c r="U39" s="31" t="inlineStr"/>
+      <c r="T39" s="24">
+        <f>N39+P39+R39</f>
+        <v/>
+      </c>
+      <c r="U39" s="25">
+        <f>T39-S39</f>
+        <v/>
+      </c>
+      <c r="V39" s="31" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="20" t="inlineStr">
@@ -3297,50 +3425,54 @@
         <f>G40-F40</f>
         <v/>
       </c>
-      <c r="I40" s="26">
+      <c r="I40" s="23">
+        <f>ABS(G40-F40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="26">
         <f>IF(F40&gt;0, G40/F40, IF(G40&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J40" s="27">
-        <f>IF(F40=0, IF(G40=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G40-F40)/F40))</f>
-        <v/>
-      </c>
-      <c r="K40" s="28" t="inlineStr">
+      <c r="K40" s="27">
+        <f>IF(F40&gt;0, 1.0 - (I40/F40), IF(G40=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" s="23">
-        <f>L40+N40+P40</f>
-        <v/>
-      </c>
-      <c r="S40" s="24">
+      <c r="M40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" s="23">
         <f>M40+O40+Q40</f>
         <v/>
       </c>
-      <c r="T40" s="25">
-        <f>S40-R40</f>
-        <v/>
-      </c>
-      <c r="U40" s="31" t="inlineStr"/>
+      <c r="T40" s="24">
+        <f>N40+P40+R40</f>
+        <v/>
+      </c>
+      <c r="U40" s="25">
+        <f>T40-S40</f>
+        <v/>
+      </c>
+      <c r="V40" s="31" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="20" t="inlineStr">
@@ -3373,46 +3505,50 @@
         <f>G41-F41</f>
         <v/>
       </c>
-      <c r="I41" s="26">
+      <c r="I41" s="23">
+        <f>ABS(G41-F41)</f>
+        <v/>
+      </c>
+      <c r="J41" s="26">
         <f>IF(F41&gt;0, G41/F41, IF(G41&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J41" s="27">
-        <f>IF(F41=0, IF(G41=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G41-F41)/F41))</f>
-        <v/>
-      </c>
-      <c r="K41" s="28" t="inlineStr"/>
-      <c r="L41" s="29" t="n">
+      <c r="K41" s="27">
+        <f>IF(F41&gt;0, 1.0 - (I41/F41), IF(G41=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L41" s="28" t="inlineStr"/>
+      <c r="M41" s="29" t="n">
         <v>300</v>
       </c>
-      <c r="M41" s="30" t="n">
+      <c r="N41" s="30" t="n">
         <v>300</v>
       </c>
-      <c r="N41" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="23">
-        <f>L41+N41+P41</f>
-        <v/>
-      </c>
-      <c r="S41" s="24">
+      <c r="O41" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" s="23">
         <f>M41+O41+Q41</f>
         <v/>
       </c>
-      <c r="T41" s="25">
-        <f>S41-R41</f>
-        <v/>
-      </c>
-      <c r="U41" s="31" t="inlineStr"/>
+      <c r="T41" s="24">
+        <f>N41+P41+R41</f>
+        <v/>
+      </c>
+      <c r="U41" s="25">
+        <f>T41-S41</f>
+        <v/>
+      </c>
+      <c r="V41" s="31" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="20" t="inlineStr">
@@ -3445,46 +3581,50 @@
         <f>G42-F42</f>
         <v/>
       </c>
-      <c r="I42" s="26">
+      <c r="I42" s="23">
+        <f>ABS(G42-F42)</f>
+        <v/>
+      </c>
+      <c r="J42" s="26">
         <f>IF(F42&gt;0, G42/F42, IF(G42&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J42" s="27">
-        <f>IF(F42=0, IF(G42=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G42-F42)/F42))</f>
-        <v/>
-      </c>
-      <c r="K42" s="28" t="inlineStr"/>
-      <c r="L42" s="29" t="n">
+      <c r="K42" s="27">
+        <f>IF(F42&gt;0, 1.0 - (I42/F42), IF(G42=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L42" s="28" t="inlineStr"/>
+      <c r="M42" s="29" t="n">
         <v>640</v>
       </c>
-      <c r="M42" s="30" t="n">
+      <c r="N42" s="30" t="n">
         <v>640</v>
       </c>
-      <c r="N42" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" s="23">
-        <f>L42+N42+P42</f>
-        <v/>
-      </c>
-      <c r="S42" s="24">
+      <c r="O42" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" s="23">
         <f>M42+O42+Q42</f>
         <v/>
       </c>
-      <c r="T42" s="25">
-        <f>S42-R42</f>
-        <v/>
-      </c>
-      <c r="U42" s="31" t="inlineStr"/>
+      <c r="T42" s="24">
+        <f>N42+P42+R42</f>
+        <v/>
+      </c>
+      <c r="U42" s="25">
+        <f>T42-S42</f>
+        <v/>
+      </c>
+      <c r="V42" s="31" t="inlineStr"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="20" t="inlineStr">
@@ -3517,50 +3657,54 @@
         <f>G43-F43</f>
         <v/>
       </c>
-      <c r="I43" s="26">
+      <c r="I43" s="23">
+        <f>ABS(G43-F43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="26">
         <f>IF(F43&gt;0, G43/F43, IF(G43&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J43" s="27">
-        <f>IF(F43=0, IF(G43=0, 1.0, 0.0), MAX(0, 1.0 - ABS(G43-F43)/F43))</f>
-        <v/>
-      </c>
-      <c r="K43" s="28" t="inlineStr">
+      <c r="K43" s="27">
+        <f>IF(F43&gt;0, 1.0 - (I43/F43), IF(G43=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="L43" s="28" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="L43" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" s="23">
-        <f>L43+N43+P43</f>
-        <v/>
-      </c>
-      <c r="S43" s="24">
+      <c r="M43" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" s="23">
         <f>M43+O43+Q43</f>
         <v/>
       </c>
-      <c r="T43" s="25">
-        <f>S43-R43</f>
-        <v/>
-      </c>
-      <c r="U43" s="31" t="inlineStr"/>
+      <c r="T43" s="24">
+        <f>N43+P43+R43</f>
+        <v/>
+      </c>
+      <c r="U43" s="25">
+        <f>T43-S43</f>
+        <v/>
+      </c>
+      <c r="V43" s="31" t="inlineStr"/>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="B44" s="32" t="inlineStr">
@@ -3583,19 +3727,19 @@
         <f>SUM(H10:H43)</f>
         <v/>
       </c>
-      <c r="I44" s="36">
+      <c r="I44" s="34">
+        <f>SUM(I10:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="36">
         <f>IF(F44&gt;0, G44/F44, 1.0)</f>
         <v/>
       </c>
-      <c r="J44" s="36">
-        <f>IF(F44&gt;0, MAX(0, 1.0 - ABS(G44-F44)/F44), 1.0)</f>
-        <v/>
-      </c>
-      <c r="K44" s="37" t="n"/>
-      <c r="L44" s="34">
-        <f>SUM(L10:L43)</f>
-        <v/>
-      </c>
+      <c r="K44" s="36">
+        <f>IF(F44&gt;0, 1.0 - (I44/F44), 1.0)</f>
+        <v/>
+      </c>
+      <c r="L44" s="37" t="n"/>
       <c r="M44" s="34">
         <f>SUM(M10:M43)</f>
         <v/>
@@ -3624,39 +3768,43 @@
         <f>SUM(S10:S43)</f>
         <v/>
       </c>
-      <c r="T44" s="35">
+      <c r="T44" s="34">
         <f>SUM(T10:T43)</f>
         <v/>
       </c>
-      <c r="U44" s="37" t="n"/>
+      <c r="U44" s="35">
+        <f>SUM(U10:U43)</f>
+        <v/>
+      </c>
+      <c r="V44" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="B4:U4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="F8:K8"/>
-    <mergeCell ref="L8:Q8"/>
-    <mergeCell ref="B3:U3"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="B2:V2"/>
+    <mergeCell ref="S5:V5"/>
+    <mergeCell ref="M6:O6"/>
     <mergeCell ref="E6:G6"/>
-    <mergeCell ref="R5:U5"/>
     <mergeCell ref="H6:I6"/>
-    <mergeCell ref="R8:U8"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="B2:U2"/>
-    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="M8:R8"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="R6:U6"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="S8:V8"/>
+    <mergeCell ref="B4:V4"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="O6:Q6"/>
+    <mergeCell ref="F8:L8"/>
     <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B3:V3"/>
     <mergeCell ref="B44:E44"/>
+    <mergeCell ref="M5:O5"/>
     <mergeCell ref="H5:I5"/>
+    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="P6:R6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K10:K43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Motivo de Desviación" error="Por favor seleccione un motivo de la lista o escriba su comentario" type="list">
+    <dataValidation sqref="L10:L43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Motivo de Desviación" error="Por favor seleccione un motivo de la lista o escriba su comentario" type="list">
       <formula1>"Adelanto de pedidos,Atraso de pedidos,Pedido extra no previsto,Campaña habitual,Cancelado / Sin siembra,Otro motivo"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Corregir concepto de valor absoluto en desviaciones: desviacion estrictamente positiva sin inversion de signo, eliminacion de columna redundante y recalculo exacto de Forecast Accuracy
</commit_message>
<xml_diff>
--- a/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_Alfonso.xlsx
+++ b/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_Alfonso.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="+#,##0;-#,##0;0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="+#,##0;-#,##0;0"/>
     <numFmt numFmtId="166" formatCode="#,##0 &quot;u&quot;"/>
     <numFmt numFmtId="167" formatCode="+#,##0 &quot;u&quot;;-#,##0 &quot;u&quot;;0 &quot;u&quot;"/>
   </numFmts>
@@ -266,7 +266,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -296,7 +296,7 @@
     <xf numFmtId="166" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -326,9 +326,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -341,10 +338,7 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -354,6 +348,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -369,10 +366,10 @@
     <xf numFmtId="164" fontId="9" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -738,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:V44"/>
+  <dimension ref="B2:U44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -749,20 +746,19 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -775,14 +771,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DELEGADO COMERCIAL: ALFONSO | Cierre Septiembre Oficial (01/10/2026) vs Previsiones a Final de Año | Generado: 01/10/2026 10:45</t>
+          <t>DELEGADO COMERCIAL: ALFONSO | Cierre Septiembre Oficial (01/10/2026) vs Previsiones a Final de Año | Generado: 01/10/2026 14:02</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>📌 INSTRUCCIONES: 1) Revise el bloque de SEPTIEMBRE (Previsto, Real, Error Absoluto y Forecast Accuracy) e indique en col. L el motivo de la desviación (adelanto, atraso, extra). 2) En las columnas verdes (N, P, R), revise y actualice las cantidades estimadas de Octubre, Noviembre y Diciembre si prevé cambios. 3) Comente en col. V cualquier nota de campaña.</t>
+          <t>📌 INSTRUCCIONES: 1) Revise el bloque de SEPTIEMBRE (Previsto, Real, Desviación en Valor Absoluto y Forecast Accuracy) e indique en col. K el motivo de la desviación (adelanto, atraso, extra). 2) En las columnas verdes (M, O, Q), revise y actualice las cantidades estimadas de Octubre, Noviembre y Diciembre si prevé cambios. 3) Comente en col. U cualquier nota de campaña.</t>
         </is>
       </c>
     </row>
@@ -813,29 +809,28 @@
         </is>
       </c>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>PREVISIÓN INICIAL Q4 (U)</t>
         </is>
       </c>
+      <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-      <c r="P5" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>PREVISIÓN REVISADA Q4 (U)</t>
         </is>
       </c>
+      <c r="P5" s="5" t="n"/>
       <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
-      <c r="S5" s="8" t="inlineStr">
+      <c r="R5" s="8" t="inlineStr">
         <is>
           <t>VARIACIÓN NETA Q4 (U)</t>
         </is>
       </c>
+      <c r="S5" s="5" t="n"/>
       <c r="T5" s="5" t="n"/>
       <c r="U5" s="5" t="n"/>
-      <c r="V5" s="5" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="B6" s="9">
@@ -851,35 +846,34 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="11">
-        <f>J44</f>
+        <f>I44</f>
         <v/>
       </c>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="11">
-        <f>K44</f>
+        <f>J44</f>
         <v/>
       </c>
       <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="9">
+      <c r="L6" s="9">
+        <f>R44</f>
+        <v/>
+      </c>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="n"/>
+      <c r="O6" s="10">
         <f>S44</f>
         <v/>
       </c>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-      <c r="P6" s="10">
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="12">
         <f>T44</f>
         <v/>
       </c>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="12">
-        <f>U44</f>
-        <v/>
-      </c>
+      <c r="S6" s="5" t="n"/>
       <c r="T6" s="5" t="n"/>
       <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="13" t="inlineStr">
@@ -892,12 +886,12 @@
           <t>CIERRE SEPTIEMBRE 2026 (CALIBRACIÓN Y ANÁLISIS DE EXACTITUD)</t>
         </is>
       </c>
-      <c r="M8" s="15" t="inlineStr">
+      <c r="L8" s="15" t="inlineStr">
         <is>
           <t>REVISIÓN PREVISIONES MES A MES (HASTA FINAL DE AÑO 2026)</t>
         </is>
       </c>
-      <c r="S8" s="16" t="inlineStr">
+      <c r="R8" s="16" t="inlineStr">
         <is>
           <t>IMPACTO Q4 Y JUSTIFICACIÓN</t>
         </is>
@@ -941,70 +935,65 @@
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>Error Abs. Sep (u)</t>
+          <t>% Consec.</t>
         </is>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
-          <t>% Consec.</t>
+          <t>Forecast Accuracy</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr">
         <is>
-          <t>Forecast Accuracy</t>
-        </is>
-      </c>
-      <c r="L9" s="18" t="inlineStr">
-        <is>
           <t>Comentario Sep (¿Adelanto/Atraso/Extra?)</t>
         </is>
       </c>
+      <c r="L9" s="19" t="inlineStr">
+        <is>
+          <t>Oct Anterior (u)</t>
+        </is>
+      </c>
       <c r="M9" s="19" t="inlineStr">
         <is>
-          <t>Oct Anterior (u)</t>
+          <t>Oct Revisado (u)</t>
         </is>
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Oct Revisado (u)</t>
+          <t>Nov Anterior (u)</t>
         </is>
       </c>
       <c r="O9" s="19" t="inlineStr">
         <is>
-          <t>Nov Anterior (u)</t>
+          <t>Nov Revisado (u)</t>
         </is>
       </c>
       <c r="P9" s="19" t="inlineStr">
         <is>
-          <t>Nov Revisado (u)</t>
+          <t>Dic Anterior (u)</t>
         </is>
       </c>
       <c r="Q9" s="19" t="inlineStr">
         <is>
-          <t>Dic Anterior (u)</t>
-        </is>
-      </c>
-      <c r="R9" s="19" t="inlineStr">
-        <is>
           <t>Dic Revisado (u)</t>
         </is>
       </c>
+      <c r="R9" s="17" t="inlineStr">
+        <is>
+          <t>Total Q4 Ant (u)</t>
+        </is>
+      </c>
       <c r="S9" s="17" t="inlineStr">
         <is>
-          <t>Total Q4 Ant (u)</t>
+          <t>Total Q4 Rev (u)</t>
         </is>
       </c>
       <c r="T9" s="17" t="inlineStr">
         <is>
-          <t>Total Q4 Rev (u)</t>
+          <t>Dif Q4 (u)</t>
         </is>
       </c>
       <c r="U9" s="17" t="inlineStr">
-        <is>
-          <t>Dif Q4 (u)</t>
-        </is>
-      </c>
-      <c r="V9" s="17" t="inlineStr">
         <is>
           <t>Comentarios / Justificación Q4</t>
         </is>
@@ -1026,65 +1015,61 @@
           <t>BIO0020</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>BIORAD-20, 20 L</t>
         </is>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="22" t="n">
         <v>960</v>
       </c>
-      <c r="G10" s="24" t="n">
+      <c r="G10" s="23" t="n">
         <v>1280</v>
       </c>
-      <c r="H10" s="25">
-        <f>G10-F10</f>
-        <v/>
-      </c>
-      <c r="I10" s="23">
+      <c r="H10" s="22">
         <f>ABS(G10-F10)</f>
         <v/>
       </c>
-      <c r="J10" s="26">
+      <c r="I10" s="24">
         <f>IF(F10&gt;0, G10/F10, IF(G10&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K10" s="27">
-        <f>IF(F10&gt;0, 1.0 - (I10/F10), IF(G10=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L10" s="28" t="inlineStr"/>
-      <c r="M10" s="29" t="n">
+      <c r="J10" s="25">
+        <f>IF(F10&gt;0, 1.0 - (H10/F10), IF(G10=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K10" s="26" t="inlineStr"/>
+      <c r="L10" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="N10" s="30" t="n">
+      <c r="M10" s="28" t="n">
         <v>960</v>
       </c>
-      <c r="O10" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="29" t="n">
+      <c r="N10" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="R10" s="30" t="n">
+      <c r="Q10" s="28" t="n">
         <v>960</v>
+      </c>
+      <c r="R10" s="22">
+        <f>L10+N10+P10</f>
+        <v/>
       </c>
       <c r="S10" s="23">
         <f>M10+O10+Q10</f>
         <v/>
       </c>
-      <c r="T10" s="24">
-        <f>N10+P10+R10</f>
-        <v/>
-      </c>
-      <c r="U10" s="25">
-        <f>T10-S10</f>
-        <v/>
-      </c>
-      <c r="V10" s="31" t="inlineStr"/>
+      <c r="T10" s="29">
+        <f>S10-R10</f>
+        <v/>
+      </c>
+      <c r="U10" s="30" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="20" t="inlineStr">
@@ -1102,65 +1087,61 @@
           <t>BROTA0020</t>
         </is>
       </c>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>BROTAMEC, 20 L</t>
         </is>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="22" t="n">
         <v>960</v>
       </c>
-      <c r="G11" s="24" t="n">
+      <c r="G11" s="23" t="n">
         <v>1920</v>
       </c>
-      <c r="H11" s="25">
-        <f>G11-F11</f>
-        <v/>
-      </c>
-      <c r="I11" s="23">
+      <c r="H11" s="22">
         <f>ABS(G11-F11)</f>
         <v/>
       </c>
-      <c r="J11" s="26">
+      <c r="I11" s="24">
         <f>IF(F11&gt;0, G11/F11, IF(G11&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K11" s="27">
-        <f>IF(F11&gt;0, 1.0 - (I11/F11), IF(G11=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L11" s="28" t="inlineStr"/>
-      <c r="M11" s="29" t="n">
+      <c r="J11" s="25">
+        <f>IF(F11&gt;0, 1.0 - (H11/F11), IF(G11=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K11" s="26" t="inlineStr"/>
+      <c r="L11" s="27" t="n">
         <v>920</v>
       </c>
-      <c r="N11" s="30" t="n">
+      <c r="M11" s="28" t="n">
         <v>920</v>
       </c>
-      <c r="O11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="29" t="n">
+      <c r="N11" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="R11" s="30" t="n">
+      <c r="Q11" s="28" t="n">
         <v>960</v>
+      </c>
+      <c r="R11" s="22">
+        <f>L11+N11+P11</f>
+        <v/>
       </c>
       <c r="S11" s="23">
         <f>M11+O11+Q11</f>
         <v/>
       </c>
-      <c r="T11" s="24">
-        <f>N11+P11+R11</f>
-        <v/>
-      </c>
-      <c r="U11" s="25">
-        <f>T11-S11</f>
-        <v/>
-      </c>
-      <c r="V11" s="31" t="inlineStr"/>
+      <c r="T11" s="29">
+        <f>S11-R11</f>
+        <v/>
+      </c>
+      <c r="U11" s="30" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="20" t="inlineStr">
@@ -1178,69 +1159,65 @@
           <t>C-CU0020</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>CODICOBRE, 20 L</t>
         </is>
       </c>
-      <c r="F12" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="24" t="n">
+      <c r="F12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="23" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="25">
-        <f>G12-F12</f>
-        <v/>
-      </c>
-      <c r="I12" s="23">
+      <c r="H12" s="22">
         <f>ABS(G12-F12)</f>
         <v/>
       </c>
-      <c r="J12" s="26">
+      <c r="I12" s="24">
         <f>IF(F12&gt;0, G12/F12, IF(G12&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K12" s="27">
-        <f>IF(F12&gt;0, 1.0 - (I12/F12), IF(G12=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L12" s="28" t="inlineStr">
+      <c r="J12" s="25">
+        <f>IF(F12&gt;0, 1.0 - (H12/F12), IF(G12=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K12" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="30" t="n">
-        <v>0</v>
+      <c r="L12" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="22">
+        <f>L12+N12+P12</f>
+        <v/>
       </c>
       <c r="S12" s="23">
         <f>M12+O12+Q12</f>
         <v/>
       </c>
-      <c r="T12" s="24">
-        <f>N12+P12+R12</f>
-        <v/>
-      </c>
-      <c r="U12" s="25">
-        <f>T12-S12</f>
-        <v/>
-      </c>
-      <c r="V12" s="31" t="inlineStr"/>
+      <c r="T12" s="29">
+        <f>S12-R12</f>
+        <v/>
+      </c>
+      <c r="U12" s="30" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="20" t="inlineStr">
@@ -1258,69 +1235,65 @@
           <t>C-L0020</t>
         </is>
       </c>
-      <c r="E13" s="22" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>CODIBOR-L, 20 L</t>
         </is>
       </c>
-      <c r="F13" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="24" t="n">
+      <c r="F13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="23" t="n">
         <v>200</v>
       </c>
-      <c r="H13" s="25">
-        <f>G13-F13</f>
-        <v/>
-      </c>
-      <c r="I13" s="23">
+      <c r="H13" s="22">
         <f>ABS(G13-F13)</f>
         <v/>
       </c>
-      <c r="J13" s="26">
+      <c r="I13" s="24">
         <f>IF(F13&gt;0, G13/F13, IF(G13&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K13" s="27">
-        <f>IF(F13&gt;0, 1.0 - (I13/F13), IF(G13=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L13" s="28" t="inlineStr">
+      <c r="J13" s="25">
+        <f>IF(F13&gt;0, 1.0 - (H13/F13), IF(G13=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K13" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="30" t="n">
-        <v>0</v>
+      <c r="L13" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="22">
+        <f>L13+N13+P13</f>
+        <v/>
       </c>
       <c r="S13" s="23">
         <f>M13+O13+Q13</f>
         <v/>
       </c>
-      <c r="T13" s="24">
-        <f>N13+P13+R13</f>
-        <v/>
-      </c>
-      <c r="U13" s="25">
-        <f>T13-S13</f>
-        <v/>
-      </c>
-      <c r="V13" s="31" t="inlineStr"/>
+      <c r="T13" s="29">
+        <f>S13-R13</f>
+        <v/>
+      </c>
+      <c r="U13" s="30" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="20" t="inlineStr">
@@ -1338,69 +1311,65 @@
           <t>A-50(2)0005</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>CODIORGAN-A50, 5 KG</t>
         </is>
       </c>
-      <c r="F14" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="24" t="n">
+      <c r="F14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="23" t="n">
         <v>500</v>
       </c>
-      <c r="H14" s="25">
-        <f>G14-F14</f>
-        <v/>
-      </c>
-      <c r="I14" s="23">
+      <c r="H14" s="22">
         <f>ABS(G14-F14)</f>
         <v/>
       </c>
-      <c r="J14" s="26">
+      <c r="I14" s="24">
         <f>IF(F14&gt;0, G14/F14, IF(G14&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K14" s="27">
-        <f>IF(F14&gt;0, 1.0 - (I14/F14), IF(G14=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L14" s="28" t="inlineStr">
+      <c r="J14" s="25">
+        <f>IF(F14&gt;0, 1.0 - (H14/F14), IF(G14=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K14" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="30" t="n">
-        <v>0</v>
+      <c r="L14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="22">
+        <f>L14+N14+P14</f>
+        <v/>
       </c>
       <c r="S14" s="23">
         <f>M14+O14+Q14</f>
         <v/>
       </c>
-      <c r="T14" s="24">
-        <f>N14+P14+R14</f>
-        <v/>
-      </c>
-      <c r="U14" s="25">
-        <f>T14-S14</f>
-        <v/>
-      </c>
-      <c r="V14" s="31" t="inlineStr"/>
+      <c r="T14" s="29">
+        <f>S14-R14</f>
+        <v/>
+      </c>
+      <c r="U14" s="30" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="20" t="inlineStr">
@@ -1418,69 +1387,65 @@
           <t>AGRMG0005</t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>AGROXIGREEN-MG, 5 L</t>
         </is>
       </c>
-      <c r="F15" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="24" t="n">
+      <c r="F15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="H15" s="25">
-        <f>G15-F15</f>
-        <v/>
-      </c>
-      <c r="I15" s="23">
+      <c r="H15" s="22">
         <f>ABS(G15-F15)</f>
         <v/>
       </c>
-      <c r="J15" s="26">
+      <c r="I15" s="24">
         <f>IF(F15&gt;0, G15/F15, IF(G15&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K15" s="27">
-        <f>IF(F15&gt;0, 1.0 - (I15/F15), IF(G15=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L15" s="28" t="inlineStr">
+      <c r="J15" s="25">
+        <f>IF(F15&gt;0, 1.0 - (H15/F15), IF(G15=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K15" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="30" t="n">
-        <v>0</v>
+      <c r="L15" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="22">
+        <f>L15+N15+P15</f>
+        <v/>
       </c>
       <c r="S15" s="23">
         <f>M15+O15+Q15</f>
         <v/>
       </c>
-      <c r="T15" s="24">
-        <f>N15+P15+R15</f>
-        <v/>
-      </c>
-      <c r="U15" s="25">
-        <f>T15-S15</f>
-        <v/>
-      </c>
-      <c r="V15" s="31" t="inlineStr"/>
+      <c r="T15" s="29">
+        <f>S15-R15</f>
+        <v/>
+      </c>
+      <c r="U15" s="30" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="20" t="inlineStr">
@@ -1498,69 +1463,65 @@
           <t>PT0005</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
-      <c r="F16" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="24" t="n">
+      <c r="F16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="H16" s="25">
-        <f>G16-F16</f>
-        <v/>
-      </c>
-      <c r="I16" s="23">
+      <c r="H16" s="22">
         <f>ABS(G16-F16)</f>
         <v/>
       </c>
-      <c r="J16" s="26">
+      <c r="I16" s="24">
         <f>IF(F16&gt;0, G16/F16, IF(G16&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K16" s="27">
-        <f>IF(F16&gt;0, 1.0 - (I16/F16), IF(G16=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L16" s="28" t="inlineStr">
+      <c r="J16" s="25">
+        <f>IF(F16&gt;0, 1.0 - (H16/F16), IF(G16=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K16" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="30" t="n">
-        <v>0</v>
+      <c r="L16" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="22">
+        <f>L16+N16+P16</f>
+        <v/>
       </c>
       <c r="S16" s="23">
         <f>M16+O16+Q16</f>
         <v/>
       </c>
-      <c r="T16" s="24">
-        <f>N16+P16+R16</f>
-        <v/>
-      </c>
-      <c r="U16" s="25">
-        <f>T16-S16</f>
-        <v/>
-      </c>
-      <c r="V16" s="31" t="inlineStr"/>
+      <c r="T16" s="29">
+        <f>S16-R16</f>
+        <v/>
+      </c>
+      <c r="U16" s="30" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="20" t="inlineStr">
@@ -1578,69 +1539,65 @@
           <t>A-50(2)0005</t>
         </is>
       </c>
-      <c r="E17" s="22" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>CODIORGAN-A50, 5 KG</t>
         </is>
       </c>
-      <c r="F17" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="24" t="n">
+      <c r="F17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="23" t="n">
         <v>400</v>
       </c>
-      <c r="H17" s="25">
-        <f>G17-F17</f>
-        <v/>
-      </c>
-      <c r="I17" s="23">
+      <c r="H17" s="22">
         <f>ABS(G17-F17)</f>
         <v/>
       </c>
-      <c r="J17" s="26">
+      <c r="I17" s="24">
         <f>IF(F17&gt;0, G17/F17, IF(G17&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K17" s="27">
-        <f>IF(F17&gt;0, 1.0 - (I17/F17), IF(G17=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L17" s="28" t="inlineStr">
+      <c r="J17" s="25">
+        <f>IF(F17&gt;0, 1.0 - (H17/F17), IF(G17=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K17" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="30" t="n">
-        <v>0</v>
+      <c r="L17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="22">
+        <f>L17+N17+P17</f>
+        <v/>
       </c>
       <c r="S17" s="23">
         <f>M17+O17+Q17</f>
         <v/>
       </c>
-      <c r="T17" s="24">
-        <f>N17+P17+R17</f>
-        <v/>
-      </c>
-      <c r="U17" s="25">
-        <f>T17-S17</f>
-        <v/>
-      </c>
-      <c r="V17" s="31" t="inlineStr"/>
+      <c r="T17" s="29">
+        <f>S17-R17</f>
+        <v/>
+      </c>
+      <c r="U17" s="30" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="20" t="inlineStr">
@@ -1658,65 +1615,61 @@
           <t>BIO0020</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>BIORAD-20, 20 L</t>
         </is>
       </c>
-      <c r="F18" s="23" t="n">
+      <c r="F18" s="22" t="n">
         <v>400</v>
       </c>
-      <c r="G18" s="24" t="n">
+      <c r="G18" s="23" t="n">
         <v>320</v>
       </c>
-      <c r="H18" s="25">
-        <f>G18-F18</f>
-        <v/>
-      </c>
-      <c r="I18" s="23">
+      <c r="H18" s="22">
         <f>ABS(G18-F18)</f>
         <v/>
       </c>
-      <c r="J18" s="26">
+      <c r="I18" s="24">
         <f>IF(F18&gt;0, G18/F18, IF(G18&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K18" s="27">
-        <f>IF(F18&gt;0, 1.0 - (I18/F18), IF(G18=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L18" s="28" t="inlineStr"/>
-      <c r="M18" s="29" t="n">
+      <c r="J18" s="25">
+        <f>IF(F18&gt;0, 1.0 - (H18/F18), IF(G18=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K18" s="26" t="inlineStr"/>
+      <c r="L18" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="N18" s="30" t="n">
+      <c r="M18" s="28" t="n">
         <v>300</v>
       </c>
-      <c r="O18" s="29" t="n">
+      <c r="N18" s="27" t="n">
         <v>400</v>
       </c>
-      <c r="P18" s="30" t="n">
+      <c r="O18" s="28" t="n">
         <v>400</v>
       </c>
-      <c r="Q18" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="30" t="n">
-        <v>0</v>
+      <c r="P18" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="22">
+        <f>L18+N18+P18</f>
+        <v/>
       </c>
       <c r="S18" s="23">
         <f>M18+O18+Q18</f>
         <v/>
       </c>
-      <c r="T18" s="24">
-        <f>N18+P18+R18</f>
-        <v/>
-      </c>
-      <c r="U18" s="25">
-        <f>T18-S18</f>
-        <v/>
-      </c>
-      <c r="V18" s="31" t="inlineStr"/>
+      <c r="T18" s="29">
+        <f>S18-R18</f>
+        <v/>
+      </c>
+      <c r="U18" s="30" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="20" t="inlineStr">
@@ -1734,65 +1687,61 @@
           <t>BROTA0020</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>BROTAMEC, 20 L</t>
         </is>
       </c>
-      <c r="F19" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="25">
-        <f>G19-F19</f>
-        <v/>
-      </c>
-      <c r="I19" s="23">
+      <c r="F19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="22">
         <f>ABS(G19-F19)</f>
         <v/>
       </c>
-      <c r="J19" s="26">
+      <c r="I19" s="24">
         <f>IF(F19&gt;0, G19/F19, IF(G19&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K19" s="27">
-        <f>IF(F19&gt;0, 1.0 - (I19/F19), IF(G19=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L19" s="28" t="inlineStr"/>
-      <c r="M19" s="29" t="n">
+      <c r="J19" s="25">
+        <f>IF(F19&gt;0, 1.0 - (H19/F19), IF(G19=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K19" s="26" t="inlineStr"/>
+      <c r="L19" s="27" t="n">
         <v>640</v>
       </c>
-      <c r="N19" s="30" t="n">
+      <c r="M19" s="28" t="n">
         <v>640</v>
       </c>
-      <c r="O19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="30" t="n">
-        <v>0</v>
+      <c r="N19" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="22">
+        <f>L19+N19+P19</f>
+        <v/>
       </c>
       <c r="S19" s="23">
         <f>M19+O19+Q19</f>
         <v/>
       </c>
-      <c r="T19" s="24">
-        <f>N19+P19+R19</f>
-        <v/>
-      </c>
-      <c r="U19" s="25">
-        <f>T19-S19</f>
-        <v/>
-      </c>
-      <c r="V19" s="31" t="inlineStr"/>
+      <c r="T19" s="29">
+        <f>S19-R19</f>
+        <v/>
+      </c>
+      <c r="U19" s="30" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="20" t="inlineStr">
@@ -1810,69 +1759,65 @@
           <t>A-50(2)0005</t>
         </is>
       </c>
-      <c r="E20" s="22" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>CODIORGAN A-50, 5 KG</t>
         </is>
       </c>
-      <c r="F20" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="24" t="n">
+      <c r="F20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="H20" s="25">
-        <f>G20-F20</f>
-        <v/>
-      </c>
-      <c r="I20" s="23">
+      <c r="H20" s="22">
         <f>ABS(G20-F20)</f>
         <v/>
       </c>
-      <c r="J20" s="26">
+      <c r="I20" s="24">
         <f>IF(F20&gt;0, G20/F20, IF(G20&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K20" s="27">
-        <f>IF(F20&gt;0, 1.0 - (I20/F20), IF(G20=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L20" s="28" t="inlineStr">
+      <c r="J20" s="25">
+        <f>IF(F20&gt;0, 1.0 - (H20/F20), IF(G20=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K20" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="30" t="n">
-        <v>0</v>
+      <c r="L20" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="22">
+        <f>L20+N20+P20</f>
+        <v/>
       </c>
       <c r="S20" s="23">
         <f>M20+O20+Q20</f>
         <v/>
       </c>
-      <c r="T20" s="24">
-        <f>N20+P20+R20</f>
-        <v/>
-      </c>
-      <c r="U20" s="25">
-        <f>T20-S20</f>
-        <v/>
-      </c>
-      <c r="V20" s="31" t="inlineStr"/>
+      <c r="T20" s="29">
+        <f>S20-R20</f>
+        <v/>
+      </c>
+      <c r="U20" s="30" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="20" t="inlineStr">
@@ -1890,69 +1835,65 @@
           <t>AVAN0005</t>
         </is>
       </c>
-      <c r="E21" s="22" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>FLORAMEC AVANCE, 5 L</t>
         </is>
       </c>
-      <c r="F21" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="24" t="n">
+      <c r="F21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="23" t="n">
         <v>100</v>
       </c>
-      <c r="H21" s="25">
-        <f>G21-F21</f>
-        <v/>
-      </c>
-      <c r="I21" s="23">
+      <c r="H21" s="22">
         <f>ABS(G21-F21)</f>
         <v/>
       </c>
-      <c r="J21" s="26">
+      <c r="I21" s="24">
         <f>IF(F21&gt;0, G21/F21, IF(G21&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K21" s="27">
-        <f>IF(F21&gt;0, 1.0 - (I21/F21), IF(G21=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L21" s="28" t="inlineStr">
+      <c r="J21" s="25">
+        <f>IF(F21&gt;0, 1.0 - (H21/F21), IF(G21=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K21" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="30" t="n">
-        <v>0</v>
+      <c r="L21" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="22">
+        <f>L21+N21+P21</f>
+        <v/>
       </c>
       <c r="S21" s="23">
         <f>M21+O21+Q21</f>
         <v/>
       </c>
-      <c r="T21" s="24">
-        <f>N21+P21+R21</f>
-        <v/>
-      </c>
-      <c r="U21" s="25">
-        <f>T21-S21</f>
-        <v/>
-      </c>
-      <c r="V21" s="31" t="inlineStr"/>
+      <c r="T21" s="29">
+        <f>S21-R21</f>
+        <v/>
+      </c>
+      <c r="U21" s="30" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="20" t="inlineStr">
@@ -1970,69 +1911,65 @@
           <t>C-CU0005</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>CODICOBRE, 5 L</t>
         </is>
       </c>
-      <c r="F22" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="24" t="n">
+      <c r="F22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="H22" s="25">
-        <f>G22-F22</f>
-        <v/>
-      </c>
-      <c r="I22" s="23">
+      <c r="H22" s="22">
         <f>ABS(G22-F22)</f>
         <v/>
       </c>
-      <c r="J22" s="26">
+      <c r="I22" s="24">
         <f>IF(F22&gt;0, G22/F22, IF(G22&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K22" s="27">
-        <f>IF(F22&gt;0, 1.0 - (I22/F22), IF(G22=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L22" s="28" t="inlineStr">
+      <c r="J22" s="25">
+        <f>IF(F22&gt;0, 1.0 - (H22/F22), IF(G22=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K22" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="30" t="n">
-        <v>0</v>
+      <c r="L22" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="22">
+        <f>L22+N22+P22</f>
+        <v/>
       </c>
       <c r="S22" s="23">
         <f>M22+O22+Q22</f>
         <v/>
       </c>
-      <c r="T22" s="24">
-        <f>N22+P22+R22</f>
-        <v/>
-      </c>
-      <c r="U22" s="25">
-        <f>T22-S22</f>
-        <v/>
-      </c>
-      <c r="V22" s="31" t="inlineStr"/>
+      <c r="T22" s="29">
+        <f>S22-R22</f>
+        <v/>
+      </c>
+      <c r="U22" s="30" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="20" t="inlineStr">
@@ -2050,69 +1987,65 @@
           <t>S0020</t>
         </is>
       </c>
-      <c r="E23" s="22" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>SALWAX STAR, 20 L</t>
         </is>
       </c>
-      <c r="F23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="24" t="n">
+      <c r="F23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="H23" s="25">
-        <f>G23-F23</f>
-        <v/>
-      </c>
-      <c r="I23" s="23">
+      <c r="H23" s="22">
         <f>ABS(G23-F23)</f>
         <v/>
       </c>
-      <c r="J23" s="26">
+      <c r="I23" s="24">
         <f>IF(F23&gt;0, G23/F23, IF(G23&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K23" s="27">
-        <f>IF(F23&gt;0, 1.0 - (I23/F23), IF(G23=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L23" s="28" t="inlineStr">
+      <c r="J23" s="25">
+        <f>IF(F23&gt;0, 1.0 - (H23/F23), IF(G23=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K23" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="30" t="n">
-        <v>0</v>
+      <c r="L23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="22">
+        <f>L23+N23+P23</f>
+        <v/>
       </c>
       <c r="S23" s="23">
         <f>M23+O23+Q23</f>
         <v/>
       </c>
-      <c r="T23" s="24">
-        <f>N23+P23+R23</f>
-        <v/>
-      </c>
-      <c r="U23" s="25">
-        <f>T23-S23</f>
-        <v/>
-      </c>
-      <c r="V23" s="31" t="inlineStr"/>
+      <c r="T23" s="29">
+        <f>S23-R23</f>
+        <v/>
+      </c>
+      <c r="U23" s="30" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="20" t="inlineStr">
@@ -2130,69 +2063,65 @@
           <t>AGRMG0005</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="21" t="inlineStr">
         <is>
           <t>AGROXIGREEN-MG, 5 L</t>
         </is>
       </c>
-      <c r="F24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="24" t="n">
+      <c r="F24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="H24" s="25">
-        <f>G24-F24</f>
-        <v/>
-      </c>
-      <c r="I24" s="23">
+      <c r="H24" s="22">
         <f>ABS(G24-F24)</f>
         <v/>
       </c>
-      <c r="J24" s="26">
+      <c r="I24" s="24">
         <f>IF(F24&gt;0, G24/F24, IF(G24&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K24" s="27">
-        <f>IF(F24&gt;0, 1.0 - (I24/F24), IF(G24=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L24" s="28" t="inlineStr">
+      <c r="J24" s="25">
+        <f>IF(F24&gt;0, 1.0 - (H24/F24), IF(G24=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K24" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="30" t="n">
-        <v>0</v>
+      <c r="L24" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="22">
+        <f>L24+N24+P24</f>
+        <v/>
       </c>
       <c r="S24" s="23">
         <f>M24+O24+Q24</f>
         <v/>
       </c>
-      <c r="T24" s="24">
-        <f>N24+P24+R24</f>
-        <v/>
-      </c>
-      <c r="U24" s="25">
-        <f>T24-S24</f>
-        <v/>
-      </c>
-      <c r="V24" s="31" t="inlineStr"/>
+      <c r="T24" s="29">
+        <f>S24-R24</f>
+        <v/>
+      </c>
+      <c r="U24" s="30" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="20" t="inlineStr">
@@ -2210,69 +2139,65 @@
           <t>PT0005</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
-      <c r="F25" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="24" t="n">
+      <c r="F25" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="H25" s="25">
-        <f>G25-F25</f>
-        <v/>
-      </c>
-      <c r="I25" s="23">
+      <c r="H25" s="22">
         <f>ABS(G25-F25)</f>
         <v/>
       </c>
-      <c r="J25" s="26">
+      <c r="I25" s="24">
         <f>IF(F25&gt;0, G25/F25, IF(G25&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K25" s="27">
-        <f>IF(F25&gt;0, 1.0 - (I25/F25), IF(G25=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L25" s="28" t="inlineStr">
+      <c r="J25" s="25">
+        <f>IF(F25&gt;0, 1.0 - (H25/F25), IF(G25=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K25" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="30" t="n">
-        <v>0</v>
+      <c r="L25" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="22">
+        <f>L25+N25+P25</f>
+        <v/>
       </c>
       <c r="S25" s="23">
         <f>M25+O25+Q25</f>
         <v/>
       </c>
-      <c r="T25" s="24">
-        <f>N25+P25+R25</f>
-        <v/>
-      </c>
-      <c r="U25" s="25">
-        <f>T25-S25</f>
-        <v/>
-      </c>
-      <c r="V25" s="31" t="inlineStr"/>
+      <c r="T25" s="29">
+        <f>S25-R25</f>
+        <v/>
+      </c>
+      <c r="U25" s="30" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="20" t="inlineStr">
@@ -2290,69 +2215,65 @@
           <t>A-50(2)0020</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>CODIORGAN-A50, 20 KG</t>
         </is>
       </c>
-      <c r="F26" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="24" t="n">
+      <c r="F26" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="H26" s="25">
-        <f>G26-F26</f>
-        <v/>
-      </c>
-      <c r="I26" s="23">
+      <c r="H26" s="22">
         <f>ABS(G26-F26)</f>
         <v/>
       </c>
-      <c r="J26" s="26">
+      <c r="I26" s="24">
         <f>IF(F26&gt;0, G26/F26, IF(G26&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K26" s="27">
-        <f>IF(F26&gt;0, 1.0 - (I26/F26), IF(G26=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L26" s="28" t="inlineStr">
+      <c r="J26" s="25">
+        <f>IF(F26&gt;0, 1.0 - (H26/F26), IF(G26=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K26" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="30" t="n">
-        <v>0</v>
+      <c r="L26" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="22">
+        <f>L26+N26+P26</f>
+        <v/>
       </c>
       <c r="S26" s="23">
         <f>M26+O26+Q26</f>
         <v/>
       </c>
-      <c r="T26" s="24">
-        <f>N26+P26+R26</f>
-        <v/>
-      </c>
-      <c r="U26" s="25">
-        <f>T26-S26</f>
-        <v/>
-      </c>
-      <c r="V26" s="31" t="inlineStr"/>
+      <c r="T26" s="29">
+        <f>S26-R26</f>
+        <v/>
+      </c>
+      <c r="U26" s="30" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="B27" s="20" t="inlineStr">
@@ -2370,69 +2291,65 @@
           <t>AN0005</t>
         </is>
       </c>
-      <c r="E27" s="22" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>ALCAPLANT NEW, 5 KG</t>
         </is>
       </c>
-      <c r="F27" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="24" t="n">
+      <c r="F27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="H27" s="25">
-        <f>G27-F27</f>
-        <v/>
-      </c>
-      <c r="I27" s="23">
+      <c r="H27" s="22">
         <f>ABS(G27-F27)</f>
         <v/>
       </c>
-      <c r="J27" s="26">
+      <c r="I27" s="24">
         <f>IF(F27&gt;0, G27/F27, IF(G27&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K27" s="27">
-        <f>IF(F27&gt;0, 1.0 - (I27/F27), IF(G27=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L27" s="28" t="inlineStr">
+      <c r="J27" s="25">
+        <f>IF(F27&gt;0, 1.0 - (H27/F27), IF(G27=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K27" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="30" t="n">
-        <v>0</v>
+      <c r="L27" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="22">
+        <f>L27+N27+P27</f>
+        <v/>
       </c>
       <c r="S27" s="23">
         <f>M27+O27+Q27</f>
         <v/>
       </c>
-      <c r="T27" s="24">
-        <f>N27+P27+R27</f>
-        <v/>
-      </c>
-      <c r="U27" s="25">
-        <f>T27-S27</f>
-        <v/>
-      </c>
-      <c r="V27" s="31" t="inlineStr"/>
+      <c r="T27" s="29">
+        <f>S27-R27</f>
+        <v/>
+      </c>
+      <c r="U27" s="30" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="20" t="inlineStr">
@@ -2450,69 +2367,65 @@
           <t>BR-590005</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>BR-59, 5 KG</t>
         </is>
       </c>
-      <c r="F28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="24" t="n">
+      <c r="F28" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="23" t="n">
         <v>60</v>
       </c>
-      <c r="H28" s="25">
-        <f>G28-F28</f>
-        <v/>
-      </c>
-      <c r="I28" s="23">
+      <c r="H28" s="22">
         <f>ABS(G28-F28)</f>
         <v/>
       </c>
-      <c r="J28" s="26">
+      <c r="I28" s="24">
         <f>IF(F28&gt;0, G28/F28, IF(G28&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K28" s="27">
-        <f>IF(F28&gt;0, 1.0 - (I28/F28), IF(G28=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L28" s="28" t="inlineStr">
+      <c r="J28" s="25">
+        <f>IF(F28&gt;0, 1.0 - (H28/F28), IF(G28=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K28" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="30" t="n">
-        <v>0</v>
+      <c r="L28" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="22">
+        <f>L28+N28+P28</f>
+        <v/>
       </c>
       <c r="S28" s="23">
         <f>M28+O28+Q28</f>
         <v/>
       </c>
-      <c r="T28" s="24">
-        <f>N28+P28+R28</f>
-        <v/>
-      </c>
-      <c r="U28" s="25">
-        <f>T28-S28</f>
-        <v/>
-      </c>
-      <c r="V28" s="31" t="inlineStr"/>
+      <c r="T28" s="29">
+        <f>S28-R28</f>
+        <v/>
+      </c>
+      <c r="U28" s="30" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="20" t="inlineStr">
@@ -2530,69 +2443,65 @@
           <t>BROTA0020</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>BROTAMEC, 20 L</t>
         </is>
       </c>
-      <c r="F29" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="24" t="n">
+      <c r="F29" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="H29" s="25">
-        <f>G29-F29</f>
-        <v/>
-      </c>
-      <c r="I29" s="23">
+      <c r="H29" s="22">
         <f>ABS(G29-F29)</f>
         <v/>
       </c>
-      <c r="J29" s="26">
+      <c r="I29" s="24">
         <f>IF(F29&gt;0, G29/F29, IF(G29&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K29" s="27">
-        <f>IF(F29&gt;0, 1.0 - (I29/F29), IF(G29=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L29" s="28" t="inlineStr">
+      <c r="J29" s="25">
+        <f>IF(F29&gt;0, 1.0 - (H29/F29), IF(G29=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K29" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="30" t="n">
-        <v>0</v>
+      <c r="L29" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="22">
+        <f>L29+N29+P29</f>
+        <v/>
       </c>
       <c r="S29" s="23">
         <f>M29+O29+Q29</f>
         <v/>
       </c>
-      <c r="T29" s="24">
-        <f>N29+P29+R29</f>
-        <v/>
-      </c>
-      <c r="U29" s="25">
-        <f>T29-S29</f>
-        <v/>
-      </c>
-      <c r="V29" s="31" t="inlineStr"/>
+      <c r="T29" s="29">
+        <f>S29-R29</f>
+        <v/>
+      </c>
+      <c r="U29" s="30" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="20" t="inlineStr">
@@ -2610,69 +2519,65 @@
           <t>C-CU0005</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>CODICOBRE, 5 L</t>
         </is>
       </c>
-      <c r="F30" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="24" t="n">
+      <c r="F30" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="H30" s="25">
-        <f>G30-F30</f>
-        <v/>
-      </c>
-      <c r="I30" s="23">
+      <c r="H30" s="22">
         <f>ABS(G30-F30)</f>
         <v/>
       </c>
-      <c r="J30" s="26">
+      <c r="I30" s="24">
         <f>IF(F30&gt;0, G30/F30, IF(G30&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K30" s="27">
-        <f>IF(F30&gt;0, 1.0 - (I30/F30), IF(G30=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L30" s="28" t="inlineStr">
+      <c r="J30" s="25">
+        <f>IF(F30&gt;0, 1.0 - (H30/F30), IF(G30=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K30" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M30" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="30" t="n">
-        <v>0</v>
+      <c r="L30" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="22">
+        <f>L30+N30+P30</f>
+        <v/>
       </c>
       <c r="S30" s="23">
         <f>M30+O30+Q30</f>
         <v/>
       </c>
-      <c r="T30" s="24">
-        <f>N30+P30+R30</f>
-        <v/>
-      </c>
-      <c r="U30" s="25">
-        <f>T30-S30</f>
-        <v/>
-      </c>
-      <c r="V30" s="31" t="inlineStr"/>
+      <c r="T30" s="29">
+        <f>S30-R30</f>
+        <v/>
+      </c>
+      <c r="U30" s="30" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="20" t="inlineStr">
@@ -2690,69 +2595,65 @@
           <t>PT0020</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
-      <c r="F31" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="24" t="n">
+      <c r="F31" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="H31" s="25">
-        <f>G31-F31</f>
-        <v/>
-      </c>
-      <c r="I31" s="23">
+      <c r="H31" s="22">
         <f>ABS(G31-F31)</f>
         <v/>
       </c>
-      <c r="J31" s="26">
+      <c r="I31" s="24">
         <f>IF(F31&gt;0, G31/F31, IF(G31&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K31" s="27">
-        <f>IF(F31&gt;0, 1.0 - (I31/F31), IF(G31=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L31" s="28" t="inlineStr">
+      <c r="J31" s="25">
+        <f>IF(F31&gt;0, 1.0 - (H31/F31), IF(G31=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K31" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M31" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="30" t="n">
-        <v>0</v>
+      <c r="L31" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="22">
+        <f>L31+N31+P31</f>
+        <v/>
       </c>
       <c r="S31" s="23">
         <f>M31+O31+Q31</f>
         <v/>
       </c>
-      <c r="T31" s="24">
-        <f>N31+P31+R31</f>
-        <v/>
-      </c>
-      <c r="U31" s="25">
-        <f>T31-S31</f>
-        <v/>
-      </c>
-      <c r="V31" s="31" t="inlineStr"/>
+      <c r="T31" s="29">
+        <f>S31-R31</f>
+        <v/>
+      </c>
+      <c r="U31" s="30" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="20" t="inlineStr">
@@ -2770,69 +2671,65 @@
           <t>S0020</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
+      <c r="E32" s="21" t="inlineStr">
         <is>
           <t>SALWAX STAR, 20 L</t>
         </is>
       </c>
-      <c r="F32" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="24" t="n">
+      <c r="F32" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="H32" s="25">
-        <f>G32-F32</f>
-        <v/>
-      </c>
-      <c r="I32" s="23">
+      <c r="H32" s="22">
         <f>ABS(G32-F32)</f>
         <v/>
       </c>
-      <c r="J32" s="26">
+      <c r="I32" s="24">
         <f>IF(F32&gt;0, G32/F32, IF(G32&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K32" s="27">
-        <f>IF(F32&gt;0, 1.0 - (I32/F32), IF(G32=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L32" s="28" t="inlineStr">
+      <c r="J32" s="25">
+        <f>IF(F32&gt;0, 1.0 - (H32/F32), IF(G32=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K32" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M32" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="30" t="n">
-        <v>0</v>
+      <c r="L32" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="22">
+        <f>L32+N32+P32</f>
+        <v/>
       </c>
       <c r="S32" s="23">
         <f>M32+O32+Q32</f>
         <v/>
       </c>
-      <c r="T32" s="24">
-        <f>N32+P32+R32</f>
-        <v/>
-      </c>
-      <c r="U32" s="25">
-        <f>T32-S32</f>
-        <v/>
-      </c>
-      <c r="V32" s="31" t="inlineStr"/>
+      <c r="T32" s="29">
+        <f>S32-R32</f>
+        <v/>
+      </c>
+      <c r="U32" s="30" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="20" t="inlineStr">
@@ -2850,69 +2747,65 @@
           <t>CPLUS0005</t>
         </is>
       </c>
-      <c r="E33" s="22" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>CALCIPLUS, 5 L</t>
         </is>
       </c>
-      <c r="F33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="24" t="n">
+      <c r="F33" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="H33" s="25">
-        <f>G33-F33</f>
-        <v/>
-      </c>
-      <c r="I33" s="23">
+      <c r="H33" s="22">
         <f>ABS(G33-F33)</f>
         <v/>
       </c>
-      <c r="J33" s="26">
+      <c r="I33" s="24">
         <f>IF(F33&gt;0, G33/F33, IF(G33&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K33" s="27">
-        <f>IF(F33&gt;0, 1.0 - (I33/F33), IF(G33=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L33" s="28" t="inlineStr">
+      <c r="J33" s="25">
+        <f>IF(F33&gt;0, 1.0 - (H33/F33), IF(G33=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K33" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="30" t="n">
-        <v>0</v>
+      <c r="L33" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="22">
+        <f>L33+N33+P33</f>
+        <v/>
       </c>
       <c r="S33" s="23">
         <f>M33+O33+Q33</f>
         <v/>
       </c>
-      <c r="T33" s="24">
-        <f>N33+P33+R33</f>
-        <v/>
-      </c>
-      <c r="U33" s="25">
-        <f>T33-S33</f>
-        <v/>
-      </c>
-      <c r="V33" s="31" t="inlineStr"/>
+      <c r="T33" s="29">
+        <f>S33-R33</f>
+        <v/>
+      </c>
+      <c r="U33" s="30" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="20" t="inlineStr">
@@ -2930,69 +2823,65 @@
           <t>FTK0005</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>FITOKONTROL CA FLOW, 5 KG</t>
         </is>
       </c>
-      <c r="F34" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="24" t="n">
+      <c r="F34" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="H34" s="25">
-        <f>G34-F34</f>
-        <v/>
-      </c>
-      <c r="I34" s="23">
+      <c r="H34" s="22">
         <f>ABS(G34-F34)</f>
         <v/>
       </c>
-      <c r="J34" s="26">
+      <c r="I34" s="24">
         <f>IF(F34&gt;0, G34/F34, IF(G34&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K34" s="27">
-        <f>IF(F34&gt;0, 1.0 - (I34/F34), IF(G34=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L34" s="28" t="inlineStr">
+      <c r="J34" s="25">
+        <f>IF(F34&gt;0, 1.0 - (H34/F34), IF(G34=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K34" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" s="30" t="n">
-        <v>0</v>
+      <c r="L34" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="22">
+        <f>L34+N34+P34</f>
+        <v/>
       </c>
       <c r="S34" s="23">
         <f>M34+O34+Q34</f>
         <v/>
       </c>
-      <c r="T34" s="24">
-        <f>N34+P34+R34</f>
-        <v/>
-      </c>
-      <c r="U34" s="25">
-        <f>T34-S34</f>
-        <v/>
-      </c>
-      <c r="V34" s="31" t="inlineStr"/>
+      <c r="T34" s="29">
+        <f>S34-R34</f>
+        <v/>
+      </c>
+      <c r="U34" s="30" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="20" t="inlineStr">
@@ -3010,69 +2899,65 @@
           <t>PT0001</t>
         </is>
       </c>
-      <c r="E35" s="22" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>AGROPOTASION, 1 L</t>
         </is>
       </c>
-      <c r="F35" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="24" t="n">
+      <c r="F35" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="H35" s="25">
-        <f>G35-F35</f>
-        <v/>
-      </c>
-      <c r="I35" s="23">
+      <c r="H35" s="22">
         <f>ABS(G35-F35)</f>
         <v/>
       </c>
-      <c r="J35" s="26">
+      <c r="I35" s="24">
         <f>IF(F35&gt;0, G35/F35, IF(G35&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K35" s="27">
-        <f>IF(F35&gt;0, 1.0 - (I35/F35), IF(G35=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L35" s="28" t="inlineStr">
+      <c r="J35" s="25">
+        <f>IF(F35&gt;0, 1.0 - (H35/F35), IF(G35=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K35" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="30" t="n">
-        <v>0</v>
+      <c r="L35" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="22">
+        <f>L35+N35+P35</f>
+        <v/>
       </c>
       <c r="S35" s="23">
         <f>M35+O35+Q35</f>
         <v/>
       </c>
-      <c r="T35" s="24">
-        <f>N35+P35+R35</f>
-        <v/>
-      </c>
-      <c r="U35" s="25">
-        <f>T35-S35</f>
-        <v/>
-      </c>
-      <c r="V35" s="31" t="inlineStr"/>
+      <c r="T35" s="29">
+        <f>S35-R35</f>
+        <v/>
+      </c>
+      <c r="U35" s="30" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="20" t="inlineStr">
@@ -3090,69 +2975,65 @@
           <t>PT0005</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>AGROPOTASION, 5 L</t>
         </is>
       </c>
-      <c r="F36" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="24" t="n">
+      <c r="F36" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="23" t="n">
         <v>80</v>
       </c>
-      <c r="H36" s="25">
-        <f>G36-F36</f>
-        <v/>
-      </c>
-      <c r="I36" s="23">
+      <c r="H36" s="22">
         <f>ABS(G36-F36)</f>
         <v/>
       </c>
-      <c r="J36" s="26">
+      <c r="I36" s="24">
         <f>IF(F36&gt;0, G36/F36, IF(G36&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K36" s="27">
-        <f>IF(F36&gt;0, 1.0 - (I36/F36), IF(G36=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L36" s="28" t="inlineStr">
+      <c r="J36" s="25">
+        <f>IF(F36&gt;0, 1.0 - (H36/F36), IF(G36=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K36" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M36" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N36" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" s="30" t="n">
-        <v>0</v>
+      <c r="L36" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="22">
+        <f>L36+N36+P36</f>
+        <v/>
       </c>
       <c r="S36" s="23">
         <f>M36+O36+Q36</f>
         <v/>
       </c>
-      <c r="T36" s="24">
-        <f>N36+P36+R36</f>
-        <v/>
-      </c>
-      <c r="U36" s="25">
-        <f>T36-S36</f>
-        <v/>
-      </c>
-      <c r="V36" s="31" t="inlineStr"/>
+      <c r="T36" s="29">
+        <f>S36-R36</f>
+        <v/>
+      </c>
+      <c r="U36" s="30" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="20" t="inlineStr">
@@ -3170,69 +3051,65 @@
           <t>PT0020</t>
         </is>
       </c>
-      <c r="E37" s="22" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>AGROPOTASION, 20 L</t>
         </is>
       </c>
-      <c r="F37" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="24" t="n">
+      <c r="F37" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="23" t="n">
         <v>60</v>
       </c>
-      <c r="H37" s="25">
-        <f>G37-F37</f>
-        <v/>
-      </c>
-      <c r="I37" s="23">
+      <c r="H37" s="22">
         <f>ABS(G37-F37)</f>
         <v/>
       </c>
-      <c r="J37" s="26">
+      <c r="I37" s="24">
         <f>IF(F37&gt;0, G37/F37, IF(G37&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K37" s="27">
-        <f>IF(F37&gt;0, 1.0 - (I37/F37), IF(G37=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L37" s="28" t="inlineStr">
+      <c r="J37" s="25">
+        <f>IF(F37&gt;0, 1.0 - (H37/F37), IF(G37=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K37" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M37" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" s="30" t="n">
-        <v>0</v>
+      <c r="L37" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="22">
+        <f>L37+N37+P37</f>
+        <v/>
       </c>
       <c r="S37" s="23">
         <f>M37+O37+Q37</f>
         <v/>
       </c>
-      <c r="T37" s="24">
-        <f>N37+P37+R37</f>
-        <v/>
-      </c>
-      <c r="U37" s="25">
-        <f>T37-S37</f>
-        <v/>
-      </c>
-      <c r="V37" s="31" t="inlineStr"/>
+      <c r="T37" s="29">
+        <f>S37-R37</f>
+        <v/>
+      </c>
+      <c r="U37" s="30" t="inlineStr"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="20" t="inlineStr">
@@ -3250,69 +3127,65 @@
           <t>AGXK0020</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr">
+      <c r="E38" s="21" t="inlineStr">
         <is>
           <t>AGROXILATO-K, 20 L</t>
         </is>
       </c>
-      <c r="F38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="24" t="n">
+      <c r="F38" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="23" t="n">
         <v>640</v>
       </c>
-      <c r="H38" s="25">
-        <f>G38-F38</f>
-        <v/>
-      </c>
-      <c r="I38" s="23">
+      <c r="H38" s="22">
         <f>ABS(G38-F38)</f>
         <v/>
       </c>
-      <c r="J38" s="26">
+      <c r="I38" s="24">
         <f>IF(F38&gt;0, G38/F38, IF(G38&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K38" s="27">
-        <f>IF(F38&gt;0, 1.0 - (I38/F38), IF(G38=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L38" s="28" t="inlineStr">
+      <c r="J38" s="25">
+        <f>IF(F38&gt;0, 1.0 - (H38/F38), IF(G38=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K38" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M38" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R38" s="30" t="n">
-        <v>0</v>
+      <c r="L38" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" s="22">
+        <f>L38+N38+P38</f>
+        <v/>
       </c>
       <c r="S38" s="23">
         <f>M38+O38+Q38</f>
         <v/>
       </c>
-      <c r="T38" s="24">
-        <f>N38+P38+R38</f>
-        <v/>
-      </c>
-      <c r="U38" s="25">
-        <f>T38-S38</f>
-        <v/>
-      </c>
-      <c r="V38" s="31" t="inlineStr"/>
+      <c r="T38" s="29">
+        <f>S38-R38</f>
+        <v/>
+      </c>
+      <c r="U38" s="30" t="inlineStr"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="20" t="inlineStr">
@@ -3330,69 +3203,65 @@
           <t>AN0020</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr">
+      <c r="E39" s="21" t="inlineStr">
         <is>
           <t>ALCAPLANT NEW, 20 KG</t>
         </is>
       </c>
-      <c r="F39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="24" t="n">
+      <c r="F39" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="23" t="n">
         <v>600</v>
       </c>
-      <c r="H39" s="25">
-        <f>G39-F39</f>
-        <v/>
-      </c>
-      <c r="I39" s="23">
+      <c r="H39" s="22">
         <f>ABS(G39-F39)</f>
         <v/>
       </c>
-      <c r="J39" s="26">
+      <c r="I39" s="24">
         <f>IF(F39&gt;0, G39/F39, IF(G39&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K39" s="27">
-        <f>IF(F39&gt;0, 1.0 - (I39/F39), IF(G39=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L39" s="28" t="inlineStr">
+      <c r="J39" s="25">
+        <f>IF(F39&gt;0, 1.0 - (H39/F39), IF(G39=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K39" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M39" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="30" t="n">
-        <v>0</v>
+      <c r="L39" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="22">
+        <f>L39+N39+P39</f>
+        <v/>
       </c>
       <c r="S39" s="23">
         <f>M39+O39+Q39</f>
         <v/>
       </c>
-      <c r="T39" s="24">
-        <f>N39+P39+R39</f>
-        <v/>
-      </c>
-      <c r="U39" s="25">
-        <f>T39-S39</f>
-        <v/>
-      </c>
-      <c r="V39" s="31" t="inlineStr"/>
+      <c r="T39" s="29">
+        <f>S39-R39</f>
+        <v/>
+      </c>
+      <c r="U39" s="30" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="20" t="inlineStr">
@@ -3410,69 +3279,65 @@
           <t>SS0020</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E40" s="21" t="inlineStr">
         <is>
           <t>SALWAX-CA, 20 KG</t>
         </is>
       </c>
-      <c r="F40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="24" t="n">
+      <c r="F40" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="23" t="n">
         <v>500</v>
       </c>
-      <c r="H40" s="25">
-        <f>G40-F40</f>
-        <v/>
-      </c>
-      <c r="I40" s="23">
+      <c r="H40" s="22">
         <f>ABS(G40-F40)</f>
         <v/>
       </c>
-      <c r="J40" s="26">
+      <c r="I40" s="24">
         <f>IF(F40&gt;0, G40/F40, IF(G40&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K40" s="27">
-        <f>IF(F40&gt;0, 1.0 - (I40/F40), IF(G40=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L40" s="28" t="inlineStr">
+      <c r="J40" s="25">
+        <f>IF(F40&gt;0, 1.0 - (H40/F40), IF(G40=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K40" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" s="30" t="n">
-        <v>0</v>
+      <c r="L40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="22">
+        <f>L40+N40+P40</f>
+        <v/>
       </c>
       <c r="S40" s="23">
         <f>M40+O40+Q40</f>
         <v/>
       </c>
-      <c r="T40" s="24">
-        <f>N40+P40+R40</f>
-        <v/>
-      </c>
-      <c r="U40" s="25">
-        <f>T40-S40</f>
-        <v/>
-      </c>
-      <c r="V40" s="31" t="inlineStr"/>
+      <c r="T40" s="29">
+        <f>S40-R40</f>
+        <v/>
+      </c>
+      <c r="U40" s="30" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="20" t="inlineStr">
@@ -3490,65 +3355,61 @@
           <t>BIO0020</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E41" s="21" t="inlineStr">
         <is>
           <t>BIORAD-20, 20 L</t>
         </is>
       </c>
-      <c r="F41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="25">
-        <f>G41-F41</f>
-        <v/>
-      </c>
-      <c r="I41" s="23">
+      <c r="F41" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="22">
         <f>ABS(G41-F41)</f>
         <v/>
       </c>
-      <c r="J41" s="26">
+      <c r="I41" s="24">
         <f>IF(F41&gt;0, G41/F41, IF(G41&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K41" s="27">
-        <f>IF(F41&gt;0, 1.0 - (I41/F41), IF(G41=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L41" s="28" t="inlineStr"/>
-      <c r="M41" s="29" t="n">
+      <c r="J41" s="25">
+        <f>IF(F41&gt;0, 1.0 - (H41/F41), IF(G41=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K41" s="26" t="inlineStr"/>
+      <c r="L41" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="N41" s="30" t="n">
+      <c r="M41" s="28" t="n">
         <v>300</v>
       </c>
-      <c r="O41" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="30" t="n">
-        <v>0</v>
+      <c r="N41" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="22">
+        <f>L41+N41+P41</f>
+        <v/>
       </c>
       <c r="S41" s="23">
         <f>M41+O41+Q41</f>
         <v/>
       </c>
-      <c r="T41" s="24">
-        <f>N41+P41+R41</f>
-        <v/>
-      </c>
-      <c r="U41" s="25">
-        <f>T41-S41</f>
-        <v/>
-      </c>
-      <c r="V41" s="31" t="inlineStr"/>
+      <c r="T41" s="29">
+        <f>S41-R41</f>
+        <v/>
+      </c>
+      <c r="U41" s="30" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="20" t="inlineStr">
@@ -3566,65 +3427,61 @@
           <t>BROTA0020</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E42" s="21" t="inlineStr">
         <is>
           <t>BROTAMEC, 20 L</t>
         </is>
       </c>
-      <c r="F42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="25">
-        <f>G42-F42</f>
-        <v/>
-      </c>
-      <c r="I42" s="23">
+      <c r="F42" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="22">
         <f>ABS(G42-F42)</f>
         <v/>
       </c>
-      <c r="J42" s="26">
+      <c r="I42" s="24">
         <f>IF(F42&gt;0, G42/F42, IF(G42&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K42" s="27">
-        <f>IF(F42&gt;0, 1.0 - (I42/F42), IF(G42=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L42" s="28" t="inlineStr"/>
-      <c r="M42" s="29" t="n">
+      <c r="J42" s="25">
+        <f>IF(F42&gt;0, 1.0 - (H42/F42), IF(G42=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K42" s="26" t="inlineStr"/>
+      <c r="L42" s="27" t="n">
         <v>640</v>
       </c>
-      <c r="N42" s="30" t="n">
+      <c r="M42" s="28" t="n">
         <v>640</v>
       </c>
-      <c r="O42" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" s="30" t="n">
-        <v>0</v>
+      <c r="N42" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="22">
+        <f>L42+N42+P42</f>
+        <v/>
       </c>
       <c r="S42" s="23">
         <f>M42+O42+Q42</f>
         <v/>
       </c>
-      <c r="T42" s="24">
-        <f>N42+P42+R42</f>
-        <v/>
-      </c>
-      <c r="U42" s="25">
-        <f>T42-S42</f>
-        <v/>
-      </c>
-      <c r="V42" s="31" t="inlineStr"/>
+      <c r="T42" s="29">
+        <f>S42-R42</f>
+        <v/>
+      </c>
+      <c r="U42" s="30" t="inlineStr"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="20" t="inlineStr">
@@ -3642,169 +3499,161 @@
           <t>WHITE0020</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E43" s="21" t="inlineStr">
         <is>
           <t>AGROWHITE, 20 KG</t>
         </is>
       </c>
-      <c r="F43" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="24" t="n">
+      <c r="F43" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="23" t="n">
         <v>3460</v>
       </c>
-      <c r="H43" s="25">
-        <f>G43-F43</f>
-        <v/>
-      </c>
-      <c r="I43" s="23">
+      <c r="H43" s="22">
         <f>ABS(G43-F43)</f>
         <v/>
       </c>
-      <c r="J43" s="26">
+      <c r="I43" s="24">
         <f>IF(F43&gt;0, G43/F43, IF(G43&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="K43" s="27">
-        <f>IF(F43&gt;0, 1.0 - (I43/F43), IF(G43=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="L43" s="28" t="inlineStr">
+      <c r="J43" s="25">
+        <f>IF(F43&gt;0, 1.0 - (H43/F43), IF(G43=0, 1.0, 0.0))</f>
+        <v/>
+      </c>
+      <c r="K43" s="26" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
-      <c r="M43" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="O43" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" s="30" t="n">
-        <v>0</v>
+      <c r="L43" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="22">
+        <f>L43+N43+P43</f>
+        <v/>
       </c>
       <c r="S43" s="23">
         <f>M43+O43+Q43</f>
         <v/>
       </c>
-      <c r="T43" s="24">
-        <f>N43+P43+R43</f>
-        <v/>
-      </c>
-      <c r="U43" s="25">
-        <f>T43-S43</f>
-        <v/>
-      </c>
-      <c r="V43" s="31" t="inlineStr"/>
+      <c r="T43" s="29">
+        <f>S43-R43</f>
+        <v/>
+      </c>
+      <c r="U43" s="30" t="inlineStr"/>
     </row>
     <row r="44" ht="25" customHeight="1">
-      <c r="B44" s="32" t="inlineStr">
+      <c r="B44" s="31" t="inlineStr">
         <is>
           <t>TOTAL CONSOLIDADO - ALFONSO (UNIDADES)</t>
         </is>
       </c>
-      <c r="C44" s="33" t="n"/>
-      <c r="D44" s="33" t="n"/>
-      <c r="E44" s="33" t="n"/>
-      <c r="F44" s="34">
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
+      <c r="F44" s="33">
         <f>SUM(F10:F43)</f>
         <v/>
       </c>
-      <c r="G44" s="34">
+      <c r="G44" s="33">
         <f>SUM(G10:G43)</f>
         <v/>
       </c>
-      <c r="H44" s="35">
+      <c r="H44" s="33">
         <f>SUM(H10:H43)</f>
         <v/>
       </c>
       <c r="I44" s="34">
-        <f>SUM(I10:I43)</f>
-        <v/>
-      </c>
-      <c r="J44" s="36">
         <f>IF(F44&gt;0, G44/F44, 1.0)</f>
         <v/>
       </c>
-      <c r="K44" s="36">
-        <f>IF(F44&gt;0, 1.0 - (I44/F44), 1.0)</f>
-        <v/>
-      </c>
-      <c r="L44" s="37" t="n"/>
-      <c r="M44" s="34">
+      <c r="J44" s="34">
+        <f>IF(F44&gt;0, 1.0 - (H44/F44), 1.0)</f>
+        <v/>
+      </c>
+      <c r="K44" s="35" t="n"/>
+      <c r="L44" s="33">
+        <f>SUM(L10:L43)</f>
+        <v/>
+      </c>
+      <c r="M44" s="33">
         <f>SUM(M10:M43)</f>
         <v/>
       </c>
-      <c r="N44" s="34">
+      <c r="N44" s="33">
         <f>SUM(N10:N43)</f>
         <v/>
       </c>
-      <c r="O44" s="34">
+      <c r="O44" s="33">
         <f>SUM(O10:O43)</f>
         <v/>
       </c>
-      <c r="P44" s="34">
+      <c r="P44" s="33">
         <f>SUM(P10:P43)</f>
         <v/>
       </c>
-      <c r="Q44" s="34">
+      <c r="Q44" s="33">
         <f>SUM(Q10:Q43)</f>
         <v/>
       </c>
-      <c r="R44" s="34">
+      <c r="R44" s="33">
         <f>SUM(R10:R43)</f>
         <v/>
       </c>
-      <c r="S44" s="34">
+      <c r="S44" s="33">
         <f>SUM(S10:S43)</f>
         <v/>
       </c>
-      <c r="T44" s="34">
+      <c r="T44" s="36">
         <f>SUM(T10:T43)</f>
         <v/>
       </c>
-      <c r="U44" s="35">
-        <f>SUM(U10:U43)</f>
-        <v/>
-      </c>
-      <c r="V44" s="37" t="n"/>
+      <c r="U44" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B2:V2"/>
-    <mergeCell ref="S5:V5"/>
-    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="B4:U4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="F8:K8"/>
+    <mergeCell ref="L8:Q8"/>
+    <mergeCell ref="B3:U3"/>
     <mergeCell ref="E6:G6"/>
+    <mergeCell ref="R5:U5"/>
     <mergeCell ref="H6:I6"/>
-    <mergeCell ref="M8:R8"/>
+    <mergeCell ref="R8:U8"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="B2:U2"/>
+    <mergeCell ref="L6:N6"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="P5:R5"/>
-    <mergeCell ref="S8:V8"/>
-    <mergeCell ref="B4:V4"/>
-    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="R6:U6"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="F8:L8"/>
+    <mergeCell ref="O6:Q6"/>
     <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B3:V3"/>
     <mergeCell ref="B44:E44"/>
-    <mergeCell ref="M5:O5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="P6:R6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="L10:L43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Motivo de Desviación" error="Por favor seleccione un motivo de la lista o escriba su comentario" type="list">
+    <dataValidation sqref="K10:K43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Motivo de Desviación" error="Por favor seleccione un motivo de la lista o escriba su comentario" type="list">
       <formula1>"Adelanto de pedidos,Atraso de pedidos,Pedido extra no previsto,Campaña habitual,Cancelado / Sin siembra,Otro motivo"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Eliminar columnas de Error Absoluto y Forecast Accuracy de todos los Excels (plantillas comerciales Q4, Consolidado y Seguimiento Sep)
</commit_message>
<xml_diff>
--- a/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_Alfonso.xlsx
+++ b/Revision_Previsiones_Q4_2026/Revision_Previsiones_Q4_2026_Alfonso.xlsx
@@ -266,7 +266,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -336,9 +336,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -735,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:U44"/>
+  <dimension ref="B2:T44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -747,18 +744,17 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1">
@@ -771,14 +767,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DELEGADO COMERCIAL: ALFONSO | Cierre Septiembre Oficial (01/10/2026) vs Previsiones a Final de Año | Generado: 01/10/2026 14:02</t>
+          <t>DELEGADO COMERCIAL: ALFONSO | Cierre Septiembre Oficial (01/10/2026) vs Previsiones a Final de Año | Generado: 01/10/2026 14:16</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>📌 INSTRUCCIONES: 1) Revise el bloque de SEPTIEMBRE (Previsto, Real, Desviación en Valor Absoluto y Forecast Accuracy) e indique en col. K el motivo de la desviación (adelanto, atraso, extra). 2) En las columnas verdes (M, O, Q), revise y actualice las cantidades estimadas de Octubre, Noviembre y Diciembre si prevé cambios. 3) Comente en col. U cualquier nota de campaña.</t>
+          <t>📌 INSTRUCCIONES: 1) Revise el bloque de SEPTIEMBRE (Previsto, Real, Desviación en Valor Absoluto y % Consecución) e indique en col. J el motivo de la desviación (adelanto, atraso, extra). 2) En las columnas verdes (L, N, P), revise y actualice las cantidades estimadas de Octubre, Noviembre y Diciembre si prevé cambios. 3) Comente en col. T cualquier nota de campaña.</t>
         </is>
       </c>
     </row>
@@ -803,34 +799,29 @@
         </is>
       </c>
       <c r="I5" s="5" t="n"/>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>FORECAST ACCURACY SEP (OFICIAL)</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>PREVISIÓN INICIAL Q4 (U)</t>
         </is>
       </c>
+      <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>PREVISIÓN REVISADA Q4 (U)</t>
         </is>
       </c>
+      <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
-      <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="8" t="inlineStr">
+      <c r="Q5" s="8" t="inlineStr">
         <is>
           <t>VARIACIÓN NETA Q4 (U)</t>
         </is>
       </c>
+      <c r="R5" s="5" t="n"/>
       <c r="S5" s="5" t="n"/>
       <c r="T5" s="5" t="n"/>
-      <c r="U5" s="5" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="B6" s="9">
@@ -850,30 +841,26 @@
         <v/>
       </c>
       <c r="I6" s="5" t="n"/>
-      <c r="J6" s="11">
-        <f>J44</f>
-        <v/>
-      </c>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="9">
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="9">
+        <f>Q44</f>
+        <v/>
+      </c>
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="10">
         <f>R44</f>
         <v/>
       </c>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="10">
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="12">
         <f>S44</f>
         <v/>
       </c>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="12">
-        <f>T44</f>
-        <v/>
-      </c>
+      <c r="R6" s="5" t="n"/>
       <c r="S6" s="5" t="n"/>
       <c r="T6" s="5" t="n"/>
-      <c r="U6" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="13" t="inlineStr">
@@ -883,15 +870,15 @@
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>CIERRE SEPTIEMBRE 2026 (CALIBRACIÓN Y ANÁLISIS DE EXACTITUD)</t>
-        </is>
-      </c>
-      <c r="L8" s="15" t="inlineStr">
+          <t>CIERRE SEPTIEMBRE 2026 (CALIBRACIÓN Y ANÁLISIS)</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
         <is>
           <t>REVISIÓN PREVISIONES MES A MES (HASTA FINAL DE AÑO 2026)</t>
         </is>
       </c>
-      <c r="R8" s="16" t="inlineStr">
+      <c r="Q8" s="16" t="inlineStr">
         <is>
           <t>IMPACTO Q4 Y JUSTIFICACIÓN</t>
         </is>
@@ -940,60 +927,55 @@
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
-          <t>Forecast Accuracy</t>
-        </is>
-      </c>
-      <c r="K9" s="18" t="inlineStr">
-        <is>
           <t>Comentario Sep (¿Adelanto/Atraso/Extra?)</t>
         </is>
       </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>Oct Anterior (u)</t>
+        </is>
+      </c>
       <c r="L9" s="19" t="inlineStr">
         <is>
-          <t>Oct Anterior (u)</t>
+          <t>Oct Revisado (u)</t>
         </is>
       </c>
       <c r="M9" s="19" t="inlineStr">
         <is>
-          <t>Oct Revisado (u)</t>
+          <t>Nov Anterior (u)</t>
         </is>
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Nov Anterior (u)</t>
+          <t>Nov Revisado (u)</t>
         </is>
       </c>
       <c r="O9" s="19" t="inlineStr">
         <is>
-          <t>Nov Revisado (u)</t>
+          <t>Dic Anterior (u)</t>
         </is>
       </c>
       <c r="P9" s="19" t="inlineStr">
         <is>
-          <t>Dic Anterior (u)</t>
-        </is>
-      </c>
-      <c r="Q9" s="19" t="inlineStr">
-        <is>
           <t>Dic Revisado (u)</t>
         </is>
       </c>
+      <c r="Q9" s="17" t="inlineStr">
+        <is>
+          <t>Total Q4 Ant (u)</t>
+        </is>
+      </c>
       <c r="R9" s="17" t="inlineStr">
         <is>
-          <t>Total Q4 Ant (u)</t>
+          <t>Total Q4 Rev (u)</t>
         </is>
       </c>
       <c r="S9" s="17" t="inlineStr">
         <is>
-          <t>Total Q4 Rev (u)</t>
+          <t>Dif Q4 (u)</t>
         </is>
       </c>
       <c r="T9" s="17" t="inlineStr">
-        <is>
-          <t>Dif Q4 (u)</t>
-        </is>
-      </c>
-      <c r="U9" s="17" t="inlineStr">
         <is>
           <t>Comentarios / Justificación Q4</t>
         </is>
@@ -1034,42 +1016,38 @@
         <f>IF(F10&gt;0, G10/F10, IF(G10&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J10" s="25">
-        <f>IF(F10&gt;0, 1.0 - (H10/F10), IF(G10=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K10" s="26" t="inlineStr"/>
+      <c r="J10" s="25" t="inlineStr"/>
+      <c r="K10" s="26" t="n">
+        <v>960</v>
+      </c>
       <c r="L10" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="M10" s="28" t="n">
+      <c r="M10" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="26" t="n">
         <v>960</v>
-      </c>
-      <c r="N10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="28" t="n">
-        <v>0</v>
       </c>
       <c r="P10" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="Q10" s="28" t="n">
-        <v>960</v>
-      </c>
-      <c r="R10" s="22">
+      <c r="Q10" s="22">
+        <f>K10+M10+O10</f>
+        <v/>
+      </c>
+      <c r="R10" s="23">
         <f>L10+N10+P10</f>
         <v/>
       </c>
-      <c r="S10" s="23">
-        <f>M10+O10+Q10</f>
-        <v/>
-      </c>
-      <c r="T10" s="29">
-        <f>S10-R10</f>
-        <v/>
-      </c>
-      <c r="U10" s="30" t="inlineStr"/>
+      <c r="S10" s="28">
+        <f>R10-Q10</f>
+        <v/>
+      </c>
+      <c r="T10" s="29" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="20" t="inlineStr">
@@ -1106,42 +1084,38 @@
         <f>IF(F11&gt;0, G11/F11, IF(G11&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J11" s="25">
-        <f>IF(F11&gt;0, 1.0 - (H11/F11), IF(G11=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K11" s="26" t="inlineStr"/>
+      <c r="J11" s="25" t="inlineStr"/>
+      <c r="K11" s="26" t="n">
+        <v>920</v>
+      </c>
       <c r="L11" s="27" t="n">
         <v>920</v>
       </c>
-      <c r="M11" s="28" t="n">
-        <v>920</v>
+      <c r="M11" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="N11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O11" s="28" t="n">
-        <v>0</v>
+      <c r="O11" s="26" t="n">
+        <v>960</v>
       </c>
       <c r="P11" s="27" t="n">
         <v>960</v>
       </c>
-      <c r="Q11" s="28" t="n">
-        <v>960</v>
-      </c>
-      <c r="R11" s="22">
+      <c r="Q11" s="22">
+        <f>K11+M11+O11</f>
+        <v/>
+      </c>
+      <c r="R11" s="23">
         <f>L11+N11+P11</f>
         <v/>
       </c>
-      <c r="S11" s="23">
-        <f>M11+O11+Q11</f>
-        <v/>
-      </c>
-      <c r="T11" s="29">
-        <f>S11-R11</f>
-        <v/>
-      </c>
-      <c r="U11" s="30" t="inlineStr"/>
+      <c r="S11" s="28">
+        <f>R11-Q11</f>
+        <v/>
+      </c>
+      <c r="T11" s="29" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="B12" s="20" t="inlineStr">
@@ -1178,46 +1152,42 @@
         <f>IF(F12&gt;0, G12/F12, IF(G12&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J12" s="25">
-        <f>IF(F12&gt;0, 1.0 - (H12/F12), IF(G12=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K12" s="26" t="inlineStr">
+      <c r="J12" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K12" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M12" s="28" t="n">
+      <c r="M12" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N12" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O12" s="28" t="n">
+      <c r="O12" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P12" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q12" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="22">
+      <c r="Q12" s="22">
+        <f>K12+M12+O12</f>
+        <v/>
+      </c>
+      <c r="R12" s="23">
         <f>L12+N12+P12</f>
         <v/>
       </c>
-      <c r="S12" s="23">
-        <f>M12+O12+Q12</f>
-        <v/>
-      </c>
-      <c r="T12" s="29">
-        <f>S12-R12</f>
-        <v/>
-      </c>
-      <c r="U12" s="30" t="inlineStr"/>
+      <c r="S12" s="28">
+        <f>R12-Q12</f>
+        <v/>
+      </c>
+      <c r="T12" s="29" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="B13" s="20" t="inlineStr">
@@ -1254,46 +1224,42 @@
         <f>IF(F13&gt;0, G13/F13, IF(G13&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J13" s="25">
-        <f>IF(F13&gt;0, 1.0 - (H13/F13), IF(G13=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K13" s="26" t="inlineStr">
+      <c r="J13" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K13" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L13" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M13" s="28" t="n">
+      <c r="M13" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N13" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O13" s="28" t="n">
+      <c r="O13" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P13" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q13" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="22">
+      <c r="Q13" s="22">
+        <f>K13+M13+O13</f>
+        <v/>
+      </c>
+      <c r="R13" s="23">
         <f>L13+N13+P13</f>
         <v/>
       </c>
-      <c r="S13" s="23">
-        <f>M13+O13+Q13</f>
-        <v/>
-      </c>
-      <c r="T13" s="29">
-        <f>S13-R13</f>
-        <v/>
-      </c>
-      <c r="U13" s="30" t="inlineStr"/>
+      <c r="S13" s="28">
+        <f>R13-Q13</f>
+        <v/>
+      </c>
+      <c r="T13" s="29" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="20" t="inlineStr">
@@ -1330,46 +1296,42 @@
         <f>IF(F14&gt;0, G14/F14, IF(G14&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J14" s="25">
-        <f>IF(F14&gt;0, 1.0 - (H14/F14), IF(G14=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K14" s="26" t="inlineStr">
+      <c r="J14" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K14" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L14" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M14" s="28" t="n">
+      <c r="M14" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N14" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O14" s="28" t="n">
+      <c r="O14" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P14" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="22">
+      <c r="Q14" s="22">
+        <f>K14+M14+O14</f>
+        <v/>
+      </c>
+      <c r="R14" s="23">
         <f>L14+N14+P14</f>
         <v/>
       </c>
-      <c r="S14" s="23">
-        <f>M14+O14+Q14</f>
-        <v/>
-      </c>
-      <c r="T14" s="29">
-        <f>S14-R14</f>
-        <v/>
-      </c>
-      <c r="U14" s="30" t="inlineStr"/>
+      <c r="S14" s="28">
+        <f>R14-Q14</f>
+        <v/>
+      </c>
+      <c r="T14" s="29" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="B15" s="20" t="inlineStr">
@@ -1406,46 +1368,42 @@
         <f>IF(F15&gt;0, G15/F15, IF(G15&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J15" s="25">
-        <f>IF(F15&gt;0, 1.0 - (H15/F15), IF(G15=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K15" s="26" t="inlineStr">
+      <c r="J15" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K15" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M15" s="28" t="n">
+      <c r="M15" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O15" s="28" t="n">
+      <c r="O15" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q15" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="22">
+      <c r="Q15" s="22">
+        <f>K15+M15+O15</f>
+        <v/>
+      </c>
+      <c r="R15" s="23">
         <f>L15+N15+P15</f>
         <v/>
       </c>
-      <c r="S15" s="23">
-        <f>M15+O15+Q15</f>
-        <v/>
-      </c>
-      <c r="T15" s="29">
-        <f>S15-R15</f>
-        <v/>
-      </c>
-      <c r="U15" s="30" t="inlineStr"/>
+      <c r="S15" s="28">
+        <f>R15-Q15</f>
+        <v/>
+      </c>
+      <c r="T15" s="29" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="B16" s="20" t="inlineStr">
@@ -1482,46 +1440,42 @@
         <f>IF(F16&gt;0, G16/F16, IF(G16&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J16" s="25">
-        <f>IF(F16&gt;0, 1.0 - (H16/F16), IF(G16=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K16" s="26" t="inlineStr">
+      <c r="J16" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K16" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="28" t="n">
+      <c r="M16" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O16" s="28" t="n">
+      <c r="O16" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q16" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="22">
+      <c r="Q16" s="22">
+        <f>K16+M16+O16</f>
+        <v/>
+      </c>
+      <c r="R16" s="23">
         <f>L16+N16+P16</f>
         <v/>
       </c>
-      <c r="S16" s="23">
-        <f>M16+O16+Q16</f>
-        <v/>
-      </c>
-      <c r="T16" s="29">
-        <f>S16-R16</f>
-        <v/>
-      </c>
-      <c r="U16" s="30" t="inlineStr"/>
+      <c r="S16" s="28">
+        <f>R16-Q16</f>
+        <v/>
+      </c>
+      <c r="T16" s="29" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="B17" s="20" t="inlineStr">
@@ -1558,46 +1512,42 @@
         <f>IF(F17&gt;0, G17/F17, IF(G17&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J17" s="25">
-        <f>IF(F17&gt;0, 1.0 - (H17/F17), IF(G17=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K17" s="26" t="inlineStr">
+      <c r="J17" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K17" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="28" t="n">
+      <c r="M17" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O17" s="28" t="n">
+      <c r="O17" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q17" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="22">
+      <c r="Q17" s="22">
+        <f>K17+M17+O17</f>
+        <v/>
+      </c>
+      <c r="R17" s="23">
         <f>L17+N17+P17</f>
         <v/>
       </c>
-      <c r="S17" s="23">
-        <f>M17+O17+Q17</f>
-        <v/>
-      </c>
-      <c r="T17" s="29">
-        <f>S17-R17</f>
-        <v/>
-      </c>
-      <c r="U17" s="30" t="inlineStr"/>
+      <c r="S17" s="28">
+        <f>R17-Q17</f>
+        <v/>
+      </c>
+      <c r="T17" s="29" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="B18" s="20" t="inlineStr">
@@ -1634,42 +1584,38 @@
         <f>IF(F18&gt;0, G18/F18, IF(G18&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J18" s="25">
-        <f>IF(F18&gt;0, 1.0 - (H18/F18), IF(G18=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K18" s="26" t="inlineStr"/>
+      <c r="J18" s="25" t="inlineStr"/>
+      <c r="K18" s="26" t="n">
+        <v>300</v>
+      </c>
       <c r="L18" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="M18" s="28" t="n">
-        <v>300</v>
+      <c r="M18" s="26" t="n">
+        <v>400</v>
       </c>
       <c r="N18" s="27" t="n">
         <v>400</v>
       </c>
-      <c r="O18" s="28" t="n">
-        <v>400</v>
+      <c r="O18" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="P18" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q18" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="22">
+      <c r="Q18" s="22">
+        <f>K18+M18+O18</f>
+        <v/>
+      </c>
+      <c r="R18" s="23">
         <f>L18+N18+P18</f>
         <v/>
       </c>
-      <c r="S18" s="23">
-        <f>M18+O18+Q18</f>
-        <v/>
-      </c>
-      <c r="T18" s="29">
-        <f>S18-R18</f>
-        <v/>
-      </c>
-      <c r="U18" s="30" t="inlineStr"/>
+      <c r="S18" s="28">
+        <f>R18-Q18</f>
+        <v/>
+      </c>
+      <c r="T18" s="29" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="B19" s="20" t="inlineStr">
@@ -1706,42 +1652,38 @@
         <f>IF(F19&gt;0, G19/F19, IF(G19&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J19" s="25">
-        <f>IF(F19&gt;0, 1.0 - (H19/F19), IF(G19=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K19" s="26" t="inlineStr"/>
+      <c r="J19" s="25" t="inlineStr"/>
+      <c r="K19" s="26" t="n">
+        <v>640</v>
+      </c>
       <c r="L19" s="27" t="n">
         <v>640</v>
       </c>
-      <c r="M19" s="28" t="n">
-        <v>640</v>
+      <c r="M19" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="N19" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O19" s="28" t="n">
+      <c r="O19" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P19" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q19" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="22">
+      <c r="Q19" s="22">
+        <f>K19+M19+O19</f>
+        <v/>
+      </c>
+      <c r="R19" s="23">
         <f>L19+N19+P19</f>
         <v/>
       </c>
-      <c r="S19" s="23">
-        <f>M19+O19+Q19</f>
-        <v/>
-      </c>
-      <c r="T19" s="29">
-        <f>S19-R19</f>
-        <v/>
-      </c>
-      <c r="U19" s="30" t="inlineStr"/>
+      <c r="S19" s="28">
+        <f>R19-Q19</f>
+        <v/>
+      </c>
+      <c r="T19" s="29" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="20" t="inlineStr">
@@ -1778,46 +1720,42 @@
         <f>IF(F20&gt;0, G20/F20, IF(G20&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J20" s="25">
-        <f>IF(F20&gt;0, 1.0 - (H20/F20), IF(G20=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K20" s="26" t="inlineStr">
+      <c r="J20" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K20" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L20" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M20" s="28" t="n">
+      <c r="M20" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N20" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O20" s="28" t="n">
+      <c r="O20" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P20" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="22">
+      <c r="Q20" s="22">
+        <f>K20+M20+O20</f>
+        <v/>
+      </c>
+      <c r="R20" s="23">
         <f>L20+N20+P20</f>
         <v/>
       </c>
-      <c r="S20" s="23">
-        <f>M20+O20+Q20</f>
-        <v/>
-      </c>
-      <c r="T20" s="29">
-        <f>S20-R20</f>
-        <v/>
-      </c>
-      <c r="U20" s="30" t="inlineStr"/>
+      <c r="S20" s="28">
+        <f>R20-Q20</f>
+        <v/>
+      </c>
+      <c r="T20" s="29" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="20" t="inlineStr">
@@ -1854,46 +1792,42 @@
         <f>IF(F21&gt;0, G21/F21, IF(G21&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J21" s="25">
-        <f>IF(F21&gt;0, 1.0 - (H21/F21), IF(G21=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K21" s="26" t="inlineStr">
+      <c r="J21" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K21" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L21" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M21" s="28" t="n">
+      <c r="M21" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N21" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O21" s="28" t="n">
+      <c r="O21" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P21" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q21" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="22">
+      <c r="Q21" s="22">
+        <f>K21+M21+O21</f>
+        <v/>
+      </c>
+      <c r="R21" s="23">
         <f>L21+N21+P21</f>
         <v/>
       </c>
-      <c r="S21" s="23">
-        <f>M21+O21+Q21</f>
-        <v/>
-      </c>
-      <c r="T21" s="29">
-        <f>S21-R21</f>
-        <v/>
-      </c>
-      <c r="U21" s="30" t="inlineStr"/>
+      <c r="S21" s="28">
+        <f>R21-Q21</f>
+        <v/>
+      </c>
+      <c r="T21" s="29" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="20" t="inlineStr">
@@ -1930,46 +1864,42 @@
         <f>IF(F22&gt;0, G22/F22, IF(G22&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J22" s="25">
-        <f>IF(F22&gt;0, 1.0 - (H22/F22), IF(G22=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K22" s="26" t="inlineStr">
+      <c r="J22" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K22" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L22" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M22" s="28" t="n">
+      <c r="M22" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N22" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O22" s="28" t="n">
+      <c r="O22" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P22" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q22" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="22">
+      <c r="Q22" s="22">
+        <f>K22+M22+O22</f>
+        <v/>
+      </c>
+      <c r="R22" s="23">
         <f>L22+N22+P22</f>
         <v/>
       </c>
-      <c r="S22" s="23">
-        <f>M22+O22+Q22</f>
-        <v/>
-      </c>
-      <c r="T22" s="29">
-        <f>S22-R22</f>
-        <v/>
-      </c>
-      <c r="U22" s="30" t="inlineStr"/>
+      <c r="S22" s="28">
+        <f>R22-Q22</f>
+        <v/>
+      </c>
+      <c r="T22" s="29" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="20" t="inlineStr">
@@ -2006,46 +1936,42 @@
         <f>IF(F23&gt;0, G23/F23, IF(G23&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J23" s="25">
-        <f>IF(F23&gt;0, 1.0 - (H23/F23), IF(G23=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K23" s="26" t="inlineStr">
+      <c r="J23" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K23" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L23" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M23" s="28" t="n">
+      <c r="M23" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N23" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O23" s="28" t="n">
+      <c r="O23" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P23" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q23" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="22">
+      <c r="Q23" s="22">
+        <f>K23+M23+O23</f>
+        <v/>
+      </c>
+      <c r="R23" s="23">
         <f>L23+N23+P23</f>
         <v/>
       </c>
-      <c r="S23" s="23">
-        <f>M23+O23+Q23</f>
-        <v/>
-      </c>
-      <c r="T23" s="29">
-        <f>S23-R23</f>
-        <v/>
-      </c>
-      <c r="U23" s="30" t="inlineStr"/>
+      <c r="S23" s="28">
+        <f>R23-Q23</f>
+        <v/>
+      </c>
+      <c r="T23" s="29" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="20" t="inlineStr">
@@ -2082,46 +2008,42 @@
         <f>IF(F24&gt;0, G24/F24, IF(G24&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J24" s="25">
-        <f>IF(F24&gt;0, 1.0 - (H24/F24), IF(G24=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K24" s="26" t="inlineStr">
+      <c r="J24" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K24" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L24" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M24" s="28" t="n">
+      <c r="M24" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N24" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O24" s="28" t="n">
+      <c r="O24" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P24" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q24" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="22">
+      <c r="Q24" s="22">
+        <f>K24+M24+O24</f>
+        <v/>
+      </c>
+      <c r="R24" s="23">
         <f>L24+N24+P24</f>
         <v/>
       </c>
-      <c r="S24" s="23">
-        <f>M24+O24+Q24</f>
-        <v/>
-      </c>
-      <c r="T24" s="29">
-        <f>S24-R24</f>
-        <v/>
-      </c>
-      <c r="U24" s="30" t="inlineStr"/>
+      <c r="S24" s="28">
+        <f>R24-Q24</f>
+        <v/>
+      </c>
+      <c r="T24" s="29" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="20" t="inlineStr">
@@ -2158,46 +2080,42 @@
         <f>IF(F25&gt;0, G25/F25, IF(G25&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J25" s="25">
-        <f>IF(F25&gt;0, 1.0 - (H25/F25), IF(G25=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K25" s="26" t="inlineStr">
+      <c r="J25" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K25" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L25" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M25" s="28" t="n">
+      <c r="M25" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N25" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O25" s="28" t="n">
+      <c r="O25" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P25" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="22">
+      <c r="Q25" s="22">
+        <f>K25+M25+O25</f>
+        <v/>
+      </c>
+      <c r="R25" s="23">
         <f>L25+N25+P25</f>
         <v/>
       </c>
-      <c r="S25" s="23">
-        <f>M25+O25+Q25</f>
-        <v/>
-      </c>
-      <c r="T25" s="29">
-        <f>S25-R25</f>
-        <v/>
-      </c>
-      <c r="U25" s="30" t="inlineStr"/>
+      <c r="S25" s="28">
+        <f>R25-Q25</f>
+        <v/>
+      </c>
+      <c r="T25" s="29" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="20" t="inlineStr">
@@ -2234,46 +2152,42 @@
         <f>IF(F26&gt;0, G26/F26, IF(G26&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J26" s="25">
-        <f>IF(F26&gt;0, 1.0 - (H26/F26), IF(G26=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K26" s="26" t="inlineStr">
+      <c r="J26" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K26" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L26" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M26" s="28" t="n">
+      <c r="M26" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N26" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O26" s="28" t="n">
+      <c r="O26" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P26" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q26" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="22">
+      <c r="Q26" s="22">
+        <f>K26+M26+O26</f>
+        <v/>
+      </c>
+      <c r="R26" s="23">
         <f>L26+N26+P26</f>
         <v/>
       </c>
-      <c r="S26" s="23">
-        <f>M26+O26+Q26</f>
-        <v/>
-      </c>
-      <c r="T26" s="29">
-        <f>S26-R26</f>
-        <v/>
-      </c>
-      <c r="U26" s="30" t="inlineStr"/>
+      <c r="S26" s="28">
+        <f>R26-Q26</f>
+        <v/>
+      </c>
+      <c r="T26" s="29" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="B27" s="20" t="inlineStr">
@@ -2310,46 +2224,42 @@
         <f>IF(F27&gt;0, G27/F27, IF(G27&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J27" s="25">
-        <f>IF(F27&gt;0, 1.0 - (H27/F27), IF(G27=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K27" s="26" t="inlineStr">
+      <c r="J27" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K27" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L27" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M27" s="28" t="n">
+      <c r="M27" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N27" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O27" s="28" t="n">
+      <c r="O27" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P27" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="22">
+      <c r="Q27" s="22">
+        <f>K27+M27+O27</f>
+        <v/>
+      </c>
+      <c r="R27" s="23">
         <f>L27+N27+P27</f>
         <v/>
       </c>
-      <c r="S27" s="23">
-        <f>M27+O27+Q27</f>
-        <v/>
-      </c>
-      <c r="T27" s="29">
-        <f>S27-R27</f>
-        <v/>
-      </c>
-      <c r="U27" s="30" t="inlineStr"/>
+      <c r="S27" s="28">
+        <f>R27-Q27</f>
+        <v/>
+      </c>
+      <c r="T27" s="29" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="20" t="inlineStr">
@@ -2386,46 +2296,42 @@
         <f>IF(F28&gt;0, G28/F28, IF(G28&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J28" s="25">
-        <f>IF(F28&gt;0, 1.0 - (H28/F28), IF(G28=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K28" s="26" t="inlineStr">
+      <c r="J28" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K28" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L28" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M28" s="28" t="n">
+      <c r="M28" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N28" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O28" s="28" t="n">
+      <c r="O28" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P28" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q28" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="22">
+      <c r="Q28" s="22">
+        <f>K28+M28+O28</f>
+        <v/>
+      </c>
+      <c r="R28" s="23">
         <f>L28+N28+P28</f>
         <v/>
       </c>
-      <c r="S28" s="23">
-        <f>M28+O28+Q28</f>
-        <v/>
-      </c>
-      <c r="T28" s="29">
-        <f>S28-R28</f>
-        <v/>
-      </c>
-      <c r="U28" s="30" t="inlineStr"/>
+      <c r="S28" s="28">
+        <f>R28-Q28</f>
+        <v/>
+      </c>
+      <c r="T28" s="29" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="20" t="inlineStr">
@@ -2462,46 +2368,42 @@
         <f>IF(F29&gt;0, G29/F29, IF(G29&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J29" s="25">
-        <f>IF(F29&gt;0, 1.0 - (H29/F29), IF(G29=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K29" s="26" t="inlineStr">
+      <c r="J29" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K29" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L29" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M29" s="28" t="n">
+      <c r="M29" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N29" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O29" s="28" t="n">
+      <c r="O29" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P29" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q29" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="22">
+      <c r="Q29" s="22">
+        <f>K29+M29+O29</f>
+        <v/>
+      </c>
+      <c r="R29" s="23">
         <f>L29+N29+P29</f>
         <v/>
       </c>
-      <c r="S29" s="23">
-        <f>M29+O29+Q29</f>
-        <v/>
-      </c>
-      <c r="T29" s="29">
-        <f>S29-R29</f>
-        <v/>
-      </c>
-      <c r="U29" s="30" t="inlineStr"/>
+      <c r="S29" s="28">
+        <f>R29-Q29</f>
+        <v/>
+      </c>
+      <c r="T29" s="29" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="20" t="inlineStr">
@@ -2538,46 +2440,42 @@
         <f>IF(F30&gt;0, G30/F30, IF(G30&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J30" s="25">
-        <f>IF(F30&gt;0, 1.0 - (H30/F30), IF(G30=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K30" s="26" t="inlineStr">
+      <c r="J30" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K30" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L30" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M30" s="28" t="n">
+      <c r="M30" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N30" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O30" s="28" t="n">
+      <c r="O30" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P30" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q30" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="22">
+      <c r="Q30" s="22">
+        <f>K30+M30+O30</f>
+        <v/>
+      </c>
+      <c r="R30" s="23">
         <f>L30+N30+P30</f>
         <v/>
       </c>
-      <c r="S30" s="23">
-        <f>M30+O30+Q30</f>
-        <v/>
-      </c>
-      <c r="T30" s="29">
-        <f>S30-R30</f>
-        <v/>
-      </c>
-      <c r="U30" s="30" t="inlineStr"/>
+      <c r="S30" s="28">
+        <f>R30-Q30</f>
+        <v/>
+      </c>
+      <c r="T30" s="29" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="20" t="inlineStr">
@@ -2614,46 +2512,42 @@
         <f>IF(F31&gt;0, G31/F31, IF(G31&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J31" s="25">
-        <f>IF(F31&gt;0, 1.0 - (H31/F31), IF(G31=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K31" s="26" t="inlineStr">
+      <c r="J31" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K31" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L31" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M31" s="28" t="n">
+      <c r="M31" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N31" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O31" s="28" t="n">
+      <c r="O31" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P31" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="22">
+      <c r="Q31" s="22">
+        <f>K31+M31+O31</f>
+        <v/>
+      </c>
+      <c r="R31" s="23">
         <f>L31+N31+P31</f>
         <v/>
       </c>
-      <c r="S31" s="23">
-        <f>M31+O31+Q31</f>
-        <v/>
-      </c>
-      <c r="T31" s="29">
-        <f>S31-R31</f>
-        <v/>
-      </c>
-      <c r="U31" s="30" t="inlineStr"/>
+      <c r="S31" s="28">
+        <f>R31-Q31</f>
+        <v/>
+      </c>
+      <c r="T31" s="29" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="20" t="inlineStr">
@@ -2690,46 +2584,42 @@
         <f>IF(F32&gt;0, G32/F32, IF(G32&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J32" s="25">
-        <f>IF(F32&gt;0, 1.0 - (H32/F32), IF(G32=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K32" s="26" t="inlineStr">
+      <c r="J32" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K32" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L32" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M32" s="28" t="n">
+      <c r="M32" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N32" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O32" s="28" t="n">
+      <c r="O32" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P32" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q32" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="22">
+      <c r="Q32" s="22">
+        <f>K32+M32+O32</f>
+        <v/>
+      </c>
+      <c r="R32" s="23">
         <f>L32+N32+P32</f>
         <v/>
       </c>
-      <c r="S32" s="23">
-        <f>M32+O32+Q32</f>
-        <v/>
-      </c>
-      <c r="T32" s="29">
-        <f>S32-R32</f>
-        <v/>
-      </c>
-      <c r="U32" s="30" t="inlineStr"/>
+      <c r="S32" s="28">
+        <f>R32-Q32</f>
+        <v/>
+      </c>
+      <c r="T32" s="29" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="20" t="inlineStr">
@@ -2766,46 +2656,42 @@
         <f>IF(F33&gt;0, G33/F33, IF(G33&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J33" s="25">
-        <f>IF(F33&gt;0, 1.0 - (H33/F33), IF(G33=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K33" s="26" t="inlineStr">
+      <c r="J33" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K33" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L33" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M33" s="28" t="n">
+      <c r="M33" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N33" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O33" s="28" t="n">
+      <c r="O33" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P33" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="22">
+      <c r="Q33" s="22">
+        <f>K33+M33+O33</f>
+        <v/>
+      </c>
+      <c r="R33" s="23">
         <f>L33+N33+P33</f>
         <v/>
       </c>
-      <c r="S33" s="23">
-        <f>M33+O33+Q33</f>
-        <v/>
-      </c>
-      <c r="T33" s="29">
-        <f>S33-R33</f>
-        <v/>
-      </c>
-      <c r="U33" s="30" t="inlineStr"/>
+      <c r="S33" s="28">
+        <f>R33-Q33</f>
+        <v/>
+      </c>
+      <c r="T33" s="29" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="20" t="inlineStr">
@@ -2842,46 +2728,42 @@
         <f>IF(F34&gt;0, G34/F34, IF(G34&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J34" s="25">
-        <f>IF(F34&gt;0, 1.0 - (H34/F34), IF(G34=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K34" s="26" t="inlineStr">
+      <c r="J34" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K34" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L34" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M34" s="28" t="n">
+      <c r="M34" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N34" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O34" s="28" t="n">
+      <c r="O34" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P34" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q34" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" s="22">
+      <c r="Q34" s="22">
+        <f>K34+M34+O34</f>
+        <v/>
+      </c>
+      <c r="R34" s="23">
         <f>L34+N34+P34</f>
         <v/>
       </c>
-      <c r="S34" s="23">
-        <f>M34+O34+Q34</f>
-        <v/>
-      </c>
-      <c r="T34" s="29">
-        <f>S34-R34</f>
-        <v/>
-      </c>
-      <c r="U34" s="30" t="inlineStr"/>
+      <c r="S34" s="28">
+        <f>R34-Q34</f>
+        <v/>
+      </c>
+      <c r="T34" s="29" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="20" t="inlineStr">
@@ -2918,46 +2800,42 @@
         <f>IF(F35&gt;0, G35/F35, IF(G35&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J35" s="25">
-        <f>IF(F35&gt;0, 1.0 - (H35/F35), IF(G35=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K35" s="26" t="inlineStr">
+      <c r="J35" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K35" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L35" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M35" s="28" t="n">
+      <c r="M35" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N35" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O35" s="28" t="n">
+      <c r="O35" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P35" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="22">
+      <c r="Q35" s="22">
+        <f>K35+M35+O35</f>
+        <v/>
+      </c>
+      <c r="R35" s="23">
         <f>L35+N35+P35</f>
         <v/>
       </c>
-      <c r="S35" s="23">
-        <f>M35+O35+Q35</f>
-        <v/>
-      </c>
-      <c r="T35" s="29">
-        <f>S35-R35</f>
-        <v/>
-      </c>
-      <c r="U35" s="30" t="inlineStr"/>
+      <c r="S35" s="28">
+        <f>R35-Q35</f>
+        <v/>
+      </c>
+      <c r="T35" s="29" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="20" t="inlineStr">
@@ -2994,46 +2872,42 @@
         <f>IF(F36&gt;0, G36/F36, IF(G36&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J36" s="25">
-        <f>IF(F36&gt;0, 1.0 - (H36/F36), IF(G36=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K36" s="26" t="inlineStr">
+      <c r="J36" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K36" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L36" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M36" s="28" t="n">
+      <c r="M36" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N36" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O36" s="28" t="n">
+      <c r="O36" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P36" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q36" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" s="22">
+      <c r="Q36" s="22">
+        <f>K36+M36+O36</f>
+        <v/>
+      </c>
+      <c r="R36" s="23">
         <f>L36+N36+P36</f>
         <v/>
       </c>
-      <c r="S36" s="23">
-        <f>M36+O36+Q36</f>
-        <v/>
-      </c>
-      <c r="T36" s="29">
-        <f>S36-R36</f>
-        <v/>
-      </c>
-      <c r="U36" s="30" t="inlineStr"/>
+      <c r="S36" s="28">
+        <f>R36-Q36</f>
+        <v/>
+      </c>
+      <c r="T36" s="29" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="B37" s="20" t="inlineStr">
@@ -3070,46 +2944,42 @@
         <f>IF(F37&gt;0, G37/F37, IF(G37&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J37" s="25">
-        <f>IF(F37&gt;0, 1.0 - (H37/F37), IF(G37=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K37" s="26" t="inlineStr">
+      <c r="J37" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K37" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L37" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M37" s="28" t="n">
+      <c r="M37" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N37" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O37" s="28" t="n">
+      <c r="O37" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P37" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q37" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" s="22">
+      <c r="Q37" s="22">
+        <f>K37+M37+O37</f>
+        <v/>
+      </c>
+      <c r="R37" s="23">
         <f>L37+N37+P37</f>
         <v/>
       </c>
-      <c r="S37" s="23">
-        <f>M37+O37+Q37</f>
-        <v/>
-      </c>
-      <c r="T37" s="29">
-        <f>S37-R37</f>
-        <v/>
-      </c>
-      <c r="U37" s="30" t="inlineStr"/>
+      <c r="S37" s="28">
+        <f>R37-Q37</f>
+        <v/>
+      </c>
+      <c r="T37" s="29" t="inlineStr"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="20" t="inlineStr">
@@ -3146,46 +3016,42 @@
         <f>IF(F38&gt;0, G38/F38, IF(G38&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J38" s="25">
-        <f>IF(F38&gt;0, 1.0 - (H38/F38), IF(G38=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K38" s="26" t="inlineStr">
+      <c r="J38" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K38" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L38" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M38" s="28" t="n">
+      <c r="M38" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N38" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O38" s="28" t="n">
+      <c r="O38" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P38" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R38" s="22">
+      <c r="Q38" s="22">
+        <f>K38+M38+O38</f>
+        <v/>
+      </c>
+      <c r="R38" s="23">
         <f>L38+N38+P38</f>
         <v/>
       </c>
-      <c r="S38" s="23">
-        <f>M38+O38+Q38</f>
-        <v/>
-      </c>
-      <c r="T38" s="29">
-        <f>S38-R38</f>
-        <v/>
-      </c>
-      <c r="U38" s="30" t="inlineStr"/>
+      <c r="S38" s="28">
+        <f>R38-Q38</f>
+        <v/>
+      </c>
+      <c r="T38" s="29" t="inlineStr"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="B39" s="20" t="inlineStr">
@@ -3222,46 +3088,42 @@
         <f>IF(F39&gt;0, G39/F39, IF(G39&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J39" s="25">
-        <f>IF(F39&gt;0, 1.0 - (H39/F39), IF(G39=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K39" s="26" t="inlineStr">
+      <c r="J39" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K39" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L39" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M39" s="28" t="n">
+      <c r="M39" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N39" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O39" s="28" t="n">
+      <c r="O39" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P39" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q39" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="22">
+      <c r="Q39" s="22">
+        <f>K39+M39+O39</f>
+        <v/>
+      </c>
+      <c r="R39" s="23">
         <f>L39+N39+P39</f>
         <v/>
       </c>
-      <c r="S39" s="23">
-        <f>M39+O39+Q39</f>
-        <v/>
-      </c>
-      <c r="T39" s="29">
-        <f>S39-R39</f>
-        <v/>
-      </c>
-      <c r="U39" s="30" t="inlineStr"/>
+      <c r="S39" s="28">
+        <f>R39-Q39</f>
+        <v/>
+      </c>
+      <c r="T39" s="29" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="B40" s="20" t="inlineStr">
@@ -3298,46 +3160,42 @@
         <f>IF(F40&gt;0, G40/F40, IF(G40&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J40" s="25">
-        <f>IF(F40&gt;0, 1.0 - (H40/F40), IF(G40=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K40" s="26" t="inlineStr">
+      <c r="J40" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K40" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L40" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M40" s="28" t="n">
+      <c r="M40" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N40" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O40" s="28" t="n">
+      <c r="O40" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P40" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q40" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" s="22">
+      <c r="Q40" s="22">
+        <f>K40+M40+O40</f>
+        <v/>
+      </c>
+      <c r="R40" s="23">
         <f>L40+N40+P40</f>
         <v/>
       </c>
-      <c r="S40" s="23">
-        <f>M40+O40+Q40</f>
-        <v/>
-      </c>
-      <c r="T40" s="29">
-        <f>S40-R40</f>
-        <v/>
-      </c>
-      <c r="U40" s="30" t="inlineStr"/>
+      <c r="S40" s="28">
+        <f>R40-Q40</f>
+        <v/>
+      </c>
+      <c r="T40" s="29" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="B41" s="20" t="inlineStr">
@@ -3374,42 +3232,38 @@
         <f>IF(F41&gt;0, G41/F41, IF(G41&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J41" s="25">
-        <f>IF(F41&gt;0, 1.0 - (H41/F41), IF(G41=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K41" s="26" t="inlineStr"/>
+      <c r="J41" s="25" t="inlineStr"/>
+      <c r="K41" s="26" t="n">
+        <v>300</v>
+      </c>
       <c r="L41" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="M41" s="28" t="n">
-        <v>300</v>
+      <c r="M41" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="N41" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O41" s="28" t="n">
+      <c r="O41" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P41" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q41" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="22">
+      <c r="Q41" s="22">
+        <f>K41+M41+O41</f>
+        <v/>
+      </c>
+      <c r="R41" s="23">
         <f>L41+N41+P41</f>
         <v/>
       </c>
-      <c r="S41" s="23">
-        <f>M41+O41+Q41</f>
-        <v/>
-      </c>
-      <c r="T41" s="29">
-        <f>S41-R41</f>
-        <v/>
-      </c>
-      <c r="U41" s="30" t="inlineStr"/>
+      <c r="S41" s="28">
+        <f>R41-Q41</f>
+        <v/>
+      </c>
+      <c r="T41" s="29" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="B42" s="20" t="inlineStr">
@@ -3446,42 +3300,38 @@
         <f>IF(F42&gt;0, G42/F42, IF(G42&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J42" s="25">
-        <f>IF(F42&gt;0, 1.0 - (H42/F42), IF(G42=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K42" s="26" t="inlineStr"/>
+      <c r="J42" s="25" t="inlineStr"/>
+      <c r="K42" s="26" t="n">
+        <v>640</v>
+      </c>
       <c r="L42" s="27" t="n">
         <v>640</v>
       </c>
-      <c r="M42" s="28" t="n">
-        <v>640</v>
+      <c r="M42" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="N42" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O42" s="28" t="n">
+      <c r="O42" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P42" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q42" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" s="22">
+      <c r="Q42" s="22">
+        <f>K42+M42+O42</f>
+        <v/>
+      </c>
+      <c r="R42" s="23">
         <f>L42+N42+P42</f>
         <v/>
       </c>
-      <c r="S42" s="23">
-        <f>M42+O42+Q42</f>
-        <v/>
-      </c>
-      <c r="T42" s="29">
-        <f>S42-R42</f>
-        <v/>
-      </c>
-      <c r="U42" s="30" t="inlineStr"/>
+      <c r="S42" s="28">
+        <f>R42-Q42</f>
+        <v/>
+      </c>
+      <c r="T42" s="29" t="inlineStr"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="B43" s="20" t="inlineStr">
@@ -3518,142 +3368,132 @@
         <f>IF(F43&gt;0, G43/F43, IF(G43&gt;0, 1.0, 0.0))</f>
         <v/>
       </c>
-      <c r="J43" s="25">
-        <f>IF(F43&gt;0, 1.0 - (H43/F43), IF(G43=0, 1.0, 0.0))</f>
-        <v/>
-      </c>
-      <c r="K43" s="26" t="inlineStr">
+      <c r="J43" s="25" t="inlineStr">
         <is>
           <t>Pedido extra no previsto</t>
         </is>
       </c>
+      <c r="K43" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="L43" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="M43" s="28" t="n">
+      <c r="M43" s="26" t="n">
         <v>0</v>
       </c>
       <c r="N43" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="O43" s="28" t="n">
+      <c r="O43" s="26" t="n">
         <v>0</v>
       </c>
       <c r="P43" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" s="22">
+      <c r="Q43" s="22">
+        <f>K43+M43+O43</f>
+        <v/>
+      </c>
+      <c r="R43" s="23">
         <f>L43+N43+P43</f>
         <v/>
       </c>
-      <c r="S43" s="23">
-        <f>M43+O43+Q43</f>
-        <v/>
-      </c>
-      <c r="T43" s="29">
-        <f>S43-R43</f>
-        <v/>
-      </c>
-      <c r="U43" s="30" t="inlineStr"/>
+      <c r="S43" s="28">
+        <f>R43-Q43</f>
+        <v/>
+      </c>
+      <c r="T43" s="29" t="inlineStr"/>
     </row>
     <row r="44" ht="25" customHeight="1">
-      <c r="B44" s="31" t="inlineStr">
+      <c r="B44" s="30" t="inlineStr">
         <is>
           <t>TOTAL CONSOLIDADO - ALFONSO (UNIDADES)</t>
         </is>
       </c>
-      <c r="C44" s="32" t="n"/>
-      <c r="D44" s="32" t="n"/>
-      <c r="E44" s="32" t="n"/>
-      <c r="F44" s="33">
+      <c r="C44" s="31" t="n"/>
+      <c r="D44" s="31" t="n"/>
+      <c r="E44" s="31" t="n"/>
+      <c r="F44" s="32">
         <f>SUM(F10:F43)</f>
         <v/>
       </c>
-      <c r="G44" s="33">
+      <c r="G44" s="32">
         <f>SUM(G10:G43)</f>
         <v/>
       </c>
-      <c r="H44" s="33">
+      <c r="H44" s="32">
         <f>SUM(H10:H43)</f>
         <v/>
       </c>
-      <c r="I44" s="34">
+      <c r="I44" s="33">
         <f>IF(F44&gt;0, G44/F44, 1.0)</f>
         <v/>
       </c>
-      <c r="J44" s="34">
-        <f>IF(F44&gt;0, 1.0 - (H44/F44), 1.0)</f>
-        <v/>
-      </c>
-      <c r="K44" s="35" t="n"/>
-      <c r="L44" s="33">
+      <c r="J44" s="34" t="n"/>
+      <c r="K44" s="32">
+        <f>SUM(K10:K43)</f>
+        <v/>
+      </c>
+      <c r="L44" s="32">
         <f>SUM(L10:L43)</f>
         <v/>
       </c>
-      <c r="M44" s="33">
+      <c r="M44" s="32">
         <f>SUM(M10:M43)</f>
         <v/>
       </c>
-      <c r="N44" s="33">
+      <c r="N44" s="32">
         <f>SUM(N10:N43)</f>
         <v/>
       </c>
-      <c r="O44" s="33">
+      <c r="O44" s="32">
         <f>SUM(O10:O43)</f>
         <v/>
       </c>
-      <c r="P44" s="33">
+      <c r="P44" s="32">
         <f>SUM(P10:P43)</f>
         <v/>
       </c>
-      <c r="Q44" s="33">
+      <c r="Q44" s="32">
         <f>SUM(Q10:Q43)</f>
         <v/>
       </c>
-      <c r="R44" s="33">
+      <c r="R44" s="32">
         <f>SUM(R10:R43)</f>
         <v/>
       </c>
-      <c r="S44" s="33">
+      <c r="S44" s="35">
         <f>SUM(S10:S43)</f>
         <v/>
       </c>
-      <c r="T44" s="36">
-        <f>SUM(T10:T43)</f>
-        <v/>
-      </c>
-      <c r="U44" s="35" t="n"/>
+      <c r="T44" s="34" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="B4:U4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="F8:K8"/>
-    <mergeCell ref="L8:Q8"/>
-    <mergeCell ref="B3:U3"/>
+  <mergeCells count="20">
+    <mergeCell ref="N5:P5"/>
     <mergeCell ref="E6:G6"/>
-    <mergeCell ref="R5:U5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="R8:U8"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="B2:U2"/>
-    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="K8:P8"/>
+    <mergeCell ref="B4:T4"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="F8:J8"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="B3:T3"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="R6:U6"/>
+    <mergeCell ref="Q8:T8"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="Q5:T5"/>
+    <mergeCell ref="B2:T2"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="O6:Q6"/>
     <mergeCell ref="E5:G5"/>
+    <mergeCell ref="K5:M5"/>
     <mergeCell ref="B44:E44"/>
-    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="Q6:T6"/>
+    <mergeCell ref="H6:J6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K10:K43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Motivo de Desviación" error="Por favor seleccione un motivo de la lista o escriba su comentario" type="list">
+    <dataValidation sqref="J10:J43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Motivo de Desviación" error="Por favor seleccione un motivo de la lista o escriba su comentario" type="list">
       <formula1>"Adelanto de pedidos,Atraso de pedidos,Pedido extra no previsto,Campaña habitual,Cancelado / Sin siembra,Otro motivo"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>